<commit_message>
Add proposed declaration-item split (paid vs FOC)
Paid goods and free-of-charge units cannot share a declaration item:
they carry a different valuation method (Art. 70 UCC vs Art. 74(2)(a))
and a different nature of transaction. Both are item-level fields, so
one declaration with three items is sufficient.

New "JSD polozky" sheet splits the shipment into:
  1. 84151090 paid units      492 pcs, 8 597,14 / 9 641,63 kg, 52 712,91 EUR
  2. 84151090 FOC units         6 pcs,    89,67 /   102,21 kg,    581,74 EUR
  3. 84159000 wifi modules    246 pcs,     4,00 /     4,60 kg,  2 084,28 EUR

Item weights are apportioned from the packing list by unit count.
Adds an input cell for the carrier's freight to the EU border, which
apportions across items by gross weight once available.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014P3Ppg3YXwLjMLjTUfeWQh
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
+++ b/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
@@ -9,9 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="HS Code Summary" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Line items" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="F-gas" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Kontroly &amp; poznámky" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="JSD položky" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Line items" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="F-gas" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Kontroly &amp; poznámky" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="218">
   <si>
     <t xml:space="preserve">SOUHRN HS KÓDŮ / HS CODE SUMMARY</t>
   </si>
@@ -286,6 +287,75 @@
     <t xml:space="preserve">Nezahrnuje námořní přepravné/pojištění do hranice EU – viz řádek výše.</t>
   </si>
   <si>
+    <t xml:space="preserve">NÁVRH POLOŽEK CELNÍHO PROHLÁŠENÍ / PROPOSED DECLARATION ITEMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jedno JSD, tři položky. Zboží placené a zboží zdarma (FOC) musí být SAMOSTATNÉ POLOŽKY, protože mají jinou metodu hodnocení a jiný druh obchodu – nikoli však samostatná JSD. Stejné členění platí i v případě, že by se podávala dvě JSD (pak položka 1 + 3 na jedno, položka 2 na druhé).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Přepravné do hranice EU (EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">← DOPLNIT z faktury dopravce (námořní přepravné + THC + pojištění do místa vstupu do EU). Rozvrhuje se poměrem hrubé hmotnosti. Do doplnění zůstává podíl u položek nulový.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pol. č.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faktura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Podíl přepravného (EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metoda hodnocení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Druh obchodu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-plyny (t CO2e)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní bez chladícího média a venkovní předplněné R32 (placené zboží)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAD-1271-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 – převodní hodnota dováženého zboží (čl. 70 UCC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 – koupě/prodej</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky typu split – jednotky ZDARMA (FOC UNITS 1 %), 6 ks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAD-1272-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 – převodní hodnota stejného zboží (čl. 74 odst. 2 písm. a) UCC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 – bez finanční protihodnoty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CELKEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrola: součet položek musí odpovídat listu „HS Code Summary“ – 744 ks, 8 690,81 kg netto, 9 748,44 kg brutto, celní hodnota 55 378,93 EUR (bez přepravného do EU).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hmotnosti položek 1 a 2 jsou rozpočteny z Packing Listu podle počtu kusů (jednotková hmotnost × počet kusů). Kartony jsou u těchto výrobků 1:1 s kusy, rozpočet proto vychází přesně.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metoda hodnocení a druh obchodu jsou údaje NA ÚROVNI POLOŽKY, ne celého prohlášení – proto stačí jedno JSD. Kódy druhu obchodu ověřit dle aktuálního číselníku před podáním.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-plyny se deklarují za celou zásilku dohromady (106,76 t CO2e) – oprávnění/kvóta a odkaz na prohlášení o shodě musí pokrýt položku 1 i položku 2. Při rozdělení na dvě JSD je nutné uvést na obou.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ROZPIS POLOŽEK / LINE ITEM DETAIL</t>
   </si>
   <si>
@@ -328,9 +398,6 @@
     <t xml:space="preserve">Hodnota zboží celkem (EUR)</t>
   </si>
   <si>
-    <t xml:space="preserve">FAD-1271-2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">7SP024140</t>
   </si>
   <si>
@@ -527,6 +594,12 @@
   </si>
   <si>
     <t xml:space="preserve">FAD-1273-2026 účtuje 2 117,00 EUR jako „FGAS CONTRIBUTION“ (u FOC jednotek FAD-1274-2026 18,20 EUR se slevou -100 % → 0,00 EUR). Je fakturován jako služba (reverse charge), ale fakticky jde o platbu za kvótu HFC, která je podmínkou prodeje zboží. Doporučuji ZAHRNOUT do celní hodnoty HS 84151090. Prosím o potvrzení – list „HS Code Summary“ ukazuje součet s ním i bez něj.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placené zboží vs. FOC – členění prohlášení</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zboží placené a zboží zdarma NELZE deklarovat na jedné položce: mají jinou metodu hodnocení (čl. 70 UCC vs. čl. 74 odst. 2 písm. a) UCC) a jiný druh obchodu. Obojí jsou ale údaje na úrovni POLOŽKY, ne prohlášení, takže postačí JEDNO JSD se třemi položkami – viz list „JSD položky“. Dvě samostatná JSD nejsou nutná; pokud by se přesto podávala, je nutné rozvrhnout přepravné na obě a na obou uvést pokrytí kvótou F-plynů.</t>
   </si>
   <si>
     <t xml:space="preserve">Instrukce – chybí JSD vs. T1</t>
@@ -820,7 +893,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="65">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -953,6 +1026,62 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -991,14 +1120,6 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2195,6 +2316,397 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="32" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="34"/>
+      <c r="J4" s="34"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="34"/>
+    </row>
+    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84151090")</f>
+        <v>492</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>8597.14</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>9641.63</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84151090")</f>
+        <v>52260.79</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <f aca="false">ROUND('HS Code Summary'!$C$15*H7/'Line items'!$P$18,2)</f>
+        <v>452.12</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*G7/'Line items'!$N$18,2)</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <f aca="false">H7+I7+J7</f>
+        <v>52712.91</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="N7" s="21" t="n">
+        <f aca="false">105.85</f>
+        <v>105.85</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="E8" s="40" t="n">
+        <f aca="false">SUMIFS('Line items'!$K$5:$K$17,'Line items'!$G$5:$G$17,"84151090")</f>
+        <v>6</v>
+      </c>
+      <c r="F8" s="41" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$K$5:$K$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>89.67</v>
+      </c>
+      <c r="G8" s="41" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$K$5:$K$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>102.21</v>
+      </c>
+      <c r="H8" s="41" t="n">
+        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,"84151090")</f>
+        <v>581.74</v>
+      </c>
+      <c r="I8" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="41" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*G8/'Line items'!$N$18,2)</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="42" t="n">
+        <f aca="false">H8+I8+J8</f>
+        <v>581.74</v>
+      </c>
+      <c r="L8" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="M8" s="39" t="s">
+        <v>104</v>
+      </c>
+      <c r="N8" s="43" t="n">
+        <f aca="false">0.91</f>
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84159000")</f>
+        <v>246</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84159000")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>4</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84159000")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>4.6</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84159000")</f>
+        <v>2066.4</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <f aca="false">ROUND('HS Code Summary'!$C$15*H9/'Line items'!$P$18,2)</f>
+        <v>17.88</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*G9/'Line items'!$N$18,2)</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <f aca="false">H9+I9+J9</f>
+        <v>2084.28</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="N9" s="21" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="16" t="n">
+        <f aca="false">SUM(E7:E9)</f>
+        <v>744</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <f aca="false">SUM(F7:F9)</f>
+        <v>8690.81</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <f aca="false">SUM(G7:G9)</f>
+        <v>9748.44</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <f aca="false">SUM(H7:H9)</f>
+        <v>54908.93</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <f aca="false">SUM(I7:I9)</f>
+        <v>470</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <f aca="false">SUM(J7:J9)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <f aca="false">SUM(K7:K9)</f>
+        <v>55378.93</v>
+      </c>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
+    </row>
+    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="44" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="44"/>
+    </row>
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="45" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="45"/>
+      <c r="L13" s="45"/>
+      <c r="M13" s="45"/>
+      <c r="N13" s="45"/>
+    </row>
+    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="44" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="44"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="44"/>
+      <c r="N14" s="44"/>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="46"/>
+      <c r="K15" s="46"/>
+      <c r="L15" s="46"/>
+      <c r="M15" s="46"/>
+      <c r="N15" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="E4:N4"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A13:N13"/>
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A15:N15"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:R22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2219,12 +2731,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2232,13 +2744,13 @@
         <v>25</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>27</v>
@@ -2256,31 +2768,31 @@
         <v>19</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2288,55 +2800,55 @@
         <v>42</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>103</v>
+        <v>125</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G5" s="33" t="s">
+      <c r="G5" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="34" t="n">
+      <c r="I5" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="34" t="n">
+      <c r="J5" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="K5" s="34" t="n">
+      <c r="K5" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="34" t="n">
+      <c r="L5" s="48" t="n">
         <f aca="false">J5+K5</f>
         <v>25</v>
       </c>
-      <c r="M5" s="35" t="n">
+      <c r="M5" s="49" t="n">
         <v>211.25</v>
       </c>
-      <c r="N5" s="35" t="n">
+      <c r="N5" s="49" t="n">
         <v>251.25</v>
       </c>
-      <c r="O5" s="35" t="n">
+      <c r="O5" s="49" t="n">
         <v>57.6</v>
       </c>
-      <c r="P5" s="35" t="n">
+      <c r="P5" s="49" t="n">
         <v>1440</v>
       </c>
-      <c r="Q5" s="35" t="n">
+      <c r="Q5" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R5" s="35" t="n">
+      <c r="R5" s="49" t="n">
         <f aca="false">P5+Q5</f>
         <v>1440</v>
       </c>
@@ -2346,55 +2858,55 @@
         <v>42</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>106</v>
+        <v>128</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>107</v>
+        <v>129</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G6" s="33" t="s">
+      <c r="G6" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="34" t="n">
+      <c r="I6" s="48" t="n">
         <v>64</v>
       </c>
-      <c r="J6" s="34" t="n">
+      <c r="J6" s="48" t="n">
         <v>63</v>
       </c>
-      <c r="K6" s="34" t="n">
+      <c r="K6" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="34" t="n">
+      <c r="L6" s="48" t="n">
         <f aca="false">J6+K6</f>
         <v>64</v>
       </c>
-      <c r="M6" s="35" t="n">
+      <c r="M6" s="49" t="n">
         <v>629.12</v>
       </c>
-      <c r="N6" s="35" t="n">
+      <c r="N6" s="49" t="n">
         <v>750.72</v>
       </c>
-      <c r="O6" s="35" t="n">
+      <c r="O6" s="49" t="n">
         <v>63.24</v>
       </c>
-      <c r="P6" s="35" t="n">
+      <c r="P6" s="49" t="n">
         <v>3984.12</v>
       </c>
-      <c r="Q6" s="35" t="n">
+      <c r="Q6" s="49" t="n">
         <v>63.24</v>
       </c>
-      <c r="R6" s="35" t="n">
+      <c r="R6" s="49" t="n">
         <f aca="false">P6+Q6</f>
         <v>4047.36</v>
       </c>
@@ -2404,55 +2916,55 @@
         <v>42</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>108</v>
+        <v>130</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>109</v>
+        <v>131</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="34" t="n">
+      <c r="I7" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="J7" s="34" t="n">
+      <c r="J7" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="K7" s="34" t="n">
+      <c r="K7" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="34" t="n">
+      <c r="L7" s="48" t="n">
         <f aca="false">J7+K7</f>
         <v>25</v>
       </c>
-      <c r="M7" s="35" t="n">
+      <c r="M7" s="49" t="n">
         <v>260</v>
       </c>
-      <c r="N7" s="35" t="n">
+      <c r="N7" s="49" t="n">
         <v>288.75</v>
       </c>
-      <c r="O7" s="35" t="n">
+      <c r="O7" s="49" t="n">
         <v>104.27</v>
       </c>
-      <c r="P7" s="35" t="n">
+      <c r="P7" s="49" t="n">
         <v>2606.8</v>
       </c>
-      <c r="Q7" s="35" t="n">
+      <c r="Q7" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R7" s="35" t="n">
+      <c r="R7" s="49" t="n">
         <f aca="false">P7+Q7</f>
         <v>2606.8</v>
       </c>
@@ -2462,55 +2974,55 @@
         <v>42</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>110</v>
+        <v>132</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="G8" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="34" t="n">
+      <c r="I8" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="34" t="n">
+      <c r="J8" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="K8" s="34" t="n">
+      <c r="K8" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="34" t="n">
+      <c r="L8" s="48" t="n">
         <f aca="false">J8+K8</f>
         <v>10</v>
       </c>
-      <c r="M8" s="35" t="n">
+      <c r="M8" s="49" t="n">
         <v>133</v>
       </c>
-      <c r="N8" s="35" t="n">
+      <c r="N8" s="49" t="n">
         <v>157</v>
       </c>
-      <c r="O8" s="35" t="n">
+      <c r="O8" s="49" t="n">
         <v>136.8</v>
       </c>
-      <c r="P8" s="35" t="n">
+      <c r="P8" s="49" t="n">
         <v>1368</v>
       </c>
-      <c r="Q8" s="35" t="n">
+      <c r="Q8" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R8" s="35" t="n">
+      <c r="R8" s="49" t="n">
         <f aca="false">P8+Q8</f>
         <v>1368</v>
       </c>
@@ -2520,55 +3032,55 @@
         <v>42</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>113</v>
+        <v>135</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G9" s="33" t="s">
+      <c r="G9" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I9" s="34" t="n">
+      <c r="I9" s="48" t="n">
         <v>26</v>
       </c>
-      <c r="J9" s="34" t="n">
+      <c r="J9" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="K9" s="34" t="n">
+      <c r="K9" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="34" t="n">
+      <c r="L9" s="48" t="n">
         <f aca="false">J9+K9</f>
         <v>26</v>
       </c>
-      <c r="M9" s="35" t="n">
+      <c r="M9" s="49" t="n">
         <v>200.72</v>
       </c>
-      <c r="N9" s="35" t="n">
+      <c r="N9" s="49" t="n">
         <v>242.32</v>
       </c>
-      <c r="O9" s="35" t="n">
+      <c r="O9" s="49" t="n">
         <v>57.08</v>
       </c>
-      <c r="P9" s="35" t="n">
+      <c r="P9" s="49" t="n">
         <v>1426.94</v>
       </c>
-      <c r="Q9" s="35" t="n">
+      <c r="Q9" s="49" t="n">
         <v>57.08</v>
       </c>
-      <c r="R9" s="35" t="n">
+      <c r="R9" s="49" t="n">
         <f aca="false">P9+Q9</f>
         <v>1484.02</v>
       </c>
@@ -2578,55 +3090,55 @@
         <v>42</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>114</v>
+        <v>136</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>115</v>
+        <v>137</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="34" t="n">
+      <c r="I10" s="48" t="n">
         <v>64</v>
       </c>
-      <c r="J10" s="34" t="n">
+      <c r="J10" s="48" t="n">
         <v>63</v>
       </c>
-      <c r="K10" s="34" t="n">
+      <c r="K10" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="34" t="n">
+      <c r="L10" s="48" t="n">
         <f aca="false">J10+K10</f>
         <v>64</v>
       </c>
-      <c r="M10" s="35" t="n">
+      <c r="M10" s="49" t="n">
         <v>579.84</v>
       </c>
-      <c r="N10" s="35" t="n">
+      <c r="N10" s="49" t="n">
         <v>700.16</v>
       </c>
-      <c r="O10" s="35" t="n">
+      <c r="O10" s="49" t="n">
         <v>62.21</v>
       </c>
-      <c r="P10" s="35" t="n">
+      <c r="P10" s="49" t="n">
         <v>3919.44</v>
       </c>
-      <c r="Q10" s="35" t="n">
+      <c r="Q10" s="49" t="n">
         <v>62.21</v>
       </c>
-      <c r="R10" s="35" t="n">
+      <c r="R10" s="49" t="n">
         <f aca="false">P10+Q10</f>
         <v>3981.65</v>
       </c>
@@ -2636,55 +3148,55 @@
         <v>42</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>117</v>
+        <v>139</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G11" s="33" t="s">
+      <c r="G11" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="34" t="n">
+      <c r="I11" s="48" t="n">
         <v>26</v>
       </c>
-      <c r="J11" s="34" t="n">
+      <c r="J11" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="K11" s="34" t="n">
+      <c r="K11" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="34" t="n">
+      <c r="L11" s="48" t="n">
         <f aca="false">J11+K11</f>
         <v>26</v>
       </c>
-      <c r="M11" s="35" t="n">
+      <c r="M11" s="49" t="n">
         <v>247.52</v>
       </c>
-      <c r="N11" s="35" t="n">
+      <c r="N11" s="49" t="n">
         <v>300.04</v>
       </c>
-      <c r="O11" s="35" t="n">
+      <c r="O11" s="49" t="n">
         <v>101.36</v>
       </c>
-      <c r="P11" s="35" t="n">
+      <c r="P11" s="49" t="n">
         <v>2533.89</v>
       </c>
-      <c r="Q11" s="35" t="n">
+      <c r="Q11" s="49" t="n">
         <v>103.49</v>
       </c>
-      <c r="R11" s="35" t="n">
+      <c r="R11" s="49" t="n">
         <f aca="false">P11+Q11</f>
         <v>2637.38</v>
       </c>
@@ -2694,55 +3206,55 @@
         <v>42</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>119</v>
+        <v>141</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I12" s="34" t="n">
+      <c r="I12" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="34" t="n">
+      <c r="J12" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="34" t="n">
+      <c r="K12" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="34" t="n">
+      <c r="L12" s="48" t="n">
         <f aca="false">J12+K12</f>
         <v>10</v>
       </c>
-      <c r="M12" s="35" t="n">
+      <c r="M12" s="49" t="n">
         <v>122.1</v>
       </c>
-      <c r="N12" s="35" t="n">
+      <c r="N12" s="49" t="n">
         <v>146.2</v>
       </c>
-      <c r="O12" s="35" t="n">
+      <c r="O12" s="49" t="n">
         <v>136.8</v>
       </c>
-      <c r="P12" s="35" t="n">
+      <c r="P12" s="49" t="n">
         <v>1368</v>
       </c>
-      <c r="Q12" s="35" t="n">
+      <c r="Q12" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R12" s="35" t="n">
+      <c r="R12" s="49" t="n">
         <f aca="false">P12+Q12</f>
         <v>1368</v>
       </c>
@@ -2752,55 +3264,55 @@
         <v>42</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="G13" s="33" t="s">
+      <c r="G13" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I13" s="34" t="n">
+      <c r="I13" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="J13" s="34" t="n">
+      <c r="J13" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="K13" s="34" t="n">
+      <c r="K13" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="34" t="n">
+      <c r="L13" s="48" t="n">
         <f aca="false">J13+K13</f>
         <v>50</v>
       </c>
-      <c r="M13" s="35" t="n">
+      <c r="M13" s="49" t="n">
         <v>1019</v>
       </c>
-      <c r="N13" s="35" t="n">
+      <c r="N13" s="49" t="n">
         <v>1114</v>
       </c>
-      <c r="O13" s="35" t="n">
+      <c r="O13" s="49" t="n">
         <v>109.98</v>
       </c>
-      <c r="P13" s="35" t="n">
+      <c r="P13" s="49" t="n">
         <v>5499</v>
       </c>
-      <c r="Q13" s="35" t="n">
+      <c r="Q13" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R13" s="35" t="n">
+      <c r="R13" s="49" t="n">
         <f aca="false">P13+Q13</f>
         <v>5499</v>
       </c>
@@ -2810,55 +3322,55 @@
         <v>42</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I14" s="34" t="n">
+      <c r="I14" s="48" t="n">
         <v>127</v>
       </c>
-      <c r="J14" s="34" t="n">
+      <c r="J14" s="48" t="n">
         <v>126</v>
       </c>
-      <c r="K14" s="34" t="n">
+      <c r="K14" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="34" t="n">
+      <c r="L14" s="48" t="n">
         <f aca="false">J14+K14</f>
         <v>127</v>
       </c>
-      <c r="M14" s="35" t="n">
+      <c r="M14" s="49" t="n">
         <v>2961.64</v>
       </c>
-      <c r="N14" s="35" t="n">
+      <c r="N14" s="49" t="n">
         <v>3253.74</v>
       </c>
-      <c r="O14" s="35" t="n">
+      <c r="O14" s="49" t="n">
         <v>113.1</v>
       </c>
-      <c r="P14" s="35" t="n">
+      <c r="P14" s="49" t="n">
         <v>14250.6</v>
       </c>
-      <c r="Q14" s="35" t="n">
+      <c r="Q14" s="49" t="n">
         <v>113.1</v>
       </c>
-      <c r="R14" s="35" t="n">
+      <c r="R14" s="49" t="n">
         <f aca="false">P14+Q14</f>
         <v>14363.7</v>
       </c>
@@ -2868,55 +3380,55 @@
         <v>42</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I15" s="34" t="n">
+      <c r="I15" s="48" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="34" t="n">
+      <c r="J15" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="K15" s="34" t="n">
+      <c r="K15" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="34" t="n">
+      <c r="L15" s="48" t="n">
         <f aca="false">J15+K15</f>
         <v>51</v>
       </c>
-      <c r="M15" s="35" t="n">
+      <c r="M15" s="49" t="n">
         <v>1541.22</v>
       </c>
-      <c r="N15" s="35" t="n">
+      <c r="N15" s="49" t="n">
         <v>1686.06</v>
       </c>
-      <c r="O15" s="35" t="n">
+      <c r="O15" s="49" t="n">
         <v>182.62</v>
       </c>
-      <c r="P15" s="35" t="n">
+      <c r="P15" s="49" t="n">
         <v>9131</v>
       </c>
-      <c r="Q15" s="35" t="n">
+      <c r="Q15" s="49" t="n">
         <v>182.62</v>
       </c>
-      <c r="R15" s="35" t="n">
+      <c r="R15" s="49" t="n">
         <f aca="false">P15+Q15</f>
         <v>9313.62</v>
       </c>
@@ -2926,55 +3438,55 @@
         <v>42</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>122</v>
+        <v>144</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="47" t="s">
         <v>43</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="34" t="n">
+      <c r="I16" s="48" t="n">
         <v>20</v>
       </c>
-      <c r="J16" s="34" t="n">
+      <c r="J16" s="48" t="n">
         <v>20</v>
       </c>
-      <c r="K16" s="34" t="n">
+      <c r="K16" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="34" t="n">
+      <c r="L16" s="48" t="n">
         <f aca="false">J16+K16</f>
         <v>20</v>
       </c>
-      <c r="M16" s="35" t="n">
+      <c r="M16" s="49" t="n">
         <v>781.4</v>
       </c>
-      <c r="N16" s="35" t="n">
+      <c r="N16" s="49" t="n">
         <v>853.6</v>
       </c>
-      <c r="O16" s="35" t="n">
+      <c r="O16" s="49" t="n">
         <v>236.65</v>
       </c>
-      <c r="P16" s="35" t="n">
+      <c r="P16" s="49" t="n">
         <v>4733</v>
       </c>
-      <c r="Q16" s="35" t="n">
+      <c r="Q16" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R16" s="35" t="n">
+      <c r="R16" s="49" t="n">
         <f aca="false">P16+Q16</f>
         <v>4733</v>
       </c>
@@ -2984,55 +3496,55 @@
         <v>42</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>129</v>
+        <v>151</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>53</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="G17" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="G17" s="47" t="s">
         <v>52</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="I17" s="34" t="n">
+      <c r="I17" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="34" t="n">
+      <c r="J17" s="48" t="n">
         <v>246</v>
       </c>
-      <c r="K17" s="34" t="n">
+      <c r="K17" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="34" t="n">
+      <c r="L17" s="48" t="n">
         <f aca="false">J17+K17</f>
         <v>246</v>
       </c>
-      <c r="M17" s="35" t="n">
+      <c r="M17" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="N17" s="35" t="n">
+      <c r="N17" s="49" t="n">
         <v>4.6</v>
       </c>
-      <c r="O17" s="35" t="n">
+      <c r="O17" s="49" t="n">
         <v>8.4</v>
       </c>
-      <c r="P17" s="35" t="n">
+      <c r="P17" s="49" t="n">
         <v>2066.4</v>
       </c>
-      <c r="Q17" s="35" t="n">
+      <c r="Q17" s="49" t="n">
         <v>0</v>
       </c>
-      <c r="R17" s="35" t="n">
+      <c r="R17" s="49" t="n">
         <f aca="false">P17+Q17</f>
         <v>2066.4</v>
       </c>
@@ -3048,19 +3560,19 @@
       <c r="F18" s="15"/>
       <c r="G18" s="15"/>
       <c r="H18" s="15"/>
-      <c r="I18" s="36" t="n">
+      <c r="I18" s="50" t="n">
         <f aca="false">SUM(I5:I17)</f>
         <v>499</v>
       </c>
-      <c r="J18" s="36" t="n">
+      <c r="J18" s="50" t="n">
         <f aca="false">SUM(J5:J17)</f>
         <v>738</v>
       </c>
-      <c r="K18" s="36" t="n">
+      <c r="K18" s="50" t="n">
         <f aca="false">SUM(K5:K17)</f>
         <v>6</v>
       </c>
-      <c r="L18" s="36" t="n">
+      <c r="L18" s="50" t="n">
         <f aca="false">SUM(L5:L17)</f>
         <v>744</v>
       </c>
@@ -3088,17 +3600,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>132</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>134</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -3112,7 +3624,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3134,231 +3646,231 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>135</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B3" s="37" t="n">
+        <v>159</v>
+      </c>
+      <c r="B3" s="51" t="n">
         <v>675</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="C5" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="52" t="n">
         <v>50</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="38" t="n">
+      <c r="F5" s="52" t="n">
         <f aca="false">D5+E5</f>
         <v>50</v>
       </c>
-      <c r="G5" s="39" t="n">
+      <c r="G5" s="53" t="n">
         <v>0.351</v>
       </c>
-      <c r="H5" s="39" t="n">
+      <c r="H5" s="53" t="n">
         <f aca="false">F5*G5</f>
         <v>17.55</v>
       </c>
-      <c r="I5" s="39" t="n">
+      <c r="I5" s="53" t="n">
         <f aca="false">G5/$B$3*1000</f>
         <v>0.52</v>
       </c>
-      <c r="J5" s="39" t="n">
+      <c r="J5" s="53" t="n">
         <f aca="false">F5*I5</f>
         <v>26</v>
       </c>
-      <c r="K5" s="40" t="n">
+      <c r="K5" s="54" t="n">
         <v>7.02</v>
       </c>
-      <c r="L5" s="40" t="n">
+      <c r="L5" s="54" t="n">
         <f aca="false">F5*K5</f>
         <v>351</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>123</v>
+        <v>145</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="C6" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="38" t="n">
+      <c r="D6" s="52" t="n">
         <v>126</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="E6" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="38" t="n">
+      <c r="F6" s="52" t="n">
         <f aca="false">D6+E6</f>
         <v>127</v>
       </c>
-      <c r="G6" s="39" t="n">
+      <c r="G6" s="53" t="n">
         <v>0.385</v>
       </c>
-      <c r="H6" s="39" t="n">
+      <c r="H6" s="53" t="n">
         <f aca="false">F6*G6</f>
         <v>48.895</v>
       </c>
-      <c r="I6" s="39" t="n">
+      <c r="I6" s="53" t="n">
         <f aca="false">G6/$B$3*1000</f>
         <v>0.57037037037037</v>
       </c>
-      <c r="J6" s="39" t="n">
+      <c r="J6" s="53" t="n">
         <f aca="false">F6*I6</f>
         <v>72.437037037037</v>
       </c>
-      <c r="K6" s="40" t="n">
+      <c r="K6" s="54" t="n">
         <v>7.7</v>
       </c>
-      <c r="L6" s="40" t="n">
+      <c r="L6" s="54" t="n">
         <f aca="false">F6*K6</f>
         <v>977.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="52" t="n">
         <v>50</v>
       </c>
-      <c r="E7" s="38" t="n">
+      <c r="E7" s="52" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="52" t="n">
         <f aca="false">D7+E7</f>
         <v>51</v>
       </c>
-      <c r="G7" s="39" t="n">
+      <c r="G7" s="53" t="n">
         <v>0.527</v>
       </c>
-      <c r="H7" s="39" t="n">
+      <c r="H7" s="53" t="n">
         <f aca="false">F7*G7</f>
         <v>26.877</v>
       </c>
-      <c r="I7" s="39" t="n">
+      <c r="I7" s="53" t="n">
         <f aca="false">G7/$B$3*1000</f>
         <v>0.780740740740741</v>
       </c>
-      <c r="J7" s="39" t="n">
+      <c r="J7" s="53" t="n">
         <f aca="false">F7*I7</f>
         <v>39.8177777777778</v>
       </c>
-      <c r="K7" s="40" t="n">
+      <c r="K7" s="54" t="n">
         <v>10.53</v>
       </c>
-      <c r="L7" s="40" t="n">
+      <c r="L7" s="54" t="n">
         <f aca="false">F7*K7</f>
         <v>537.03</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>128</v>
+        <v>150</v>
       </c>
       <c r="C8" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="38" t="n">
+      <c r="D8" s="52" t="n">
         <v>20</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E8" s="52" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="38" t="n">
+      <c r="F8" s="52" t="n">
         <f aca="false">D8+E8</f>
         <v>20</v>
       </c>
-      <c r="G8" s="39" t="n">
+      <c r="G8" s="53" t="n">
         <v>0.675</v>
       </c>
-      <c r="H8" s="39" t="n">
+      <c r="H8" s="53" t="n">
         <f aca="false">F8*G8</f>
         <v>13.5</v>
       </c>
-      <c r="I8" s="39" t="n">
+      <c r="I8" s="53" t="n">
         <f aca="false">G8/$B$3*1000</f>
         <v>1</v>
       </c>
-      <c r="J8" s="39" t="n">
+      <c r="J8" s="53" t="n">
         <f aca="false">F8*I8</f>
         <v>20</v>
       </c>
-      <c r="K8" s="40" t="n">
+      <c r="K8" s="54" t="n">
         <v>13.5</v>
       </c>
-      <c r="L8" s="40" t="n">
+      <c r="L8" s="54" t="n">
         <f aca="false">F8*K8</f>
         <v>270</v>
       </c>
@@ -3382,84 +3894,84 @@
         <v>248</v>
       </c>
       <c r="G9" s="15"/>
-      <c r="H9" s="41" t="n">
+      <c r="H9" s="55" t="n">
         <f aca="false">SUM(H5:H8)</f>
         <v>106.822</v>
       </c>
       <c r="I9" s="15"/>
-      <c r="J9" s="41" t="n">
+      <c r="J9" s="55" t="n">
         <f aca="false">SUM(J5:J8)</f>
         <v>158.254814814815</v>
       </c>
       <c r="K9" s="15"/>
-      <c r="L9" s="42" t="n">
+      <c r="L9" s="56" t="n">
         <f aca="false">SUM(L5:L8)</f>
         <v>2135.93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="43" t="s">
-        <v>147</v>
-      </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
+      <c r="A11" s="44" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" s="44"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
-        <v>148</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="44"/>
-      <c r="K12" s="44"/>
-      <c r="L12" s="44"/>
+      <c r="A12" s="46" t="s">
+        <v>170</v>
+      </c>
+      <c r="B12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
+      <c r="I12" s="46"/>
+      <c r="J12" s="46"/>
+      <c r="K12" s="46"/>
+      <c r="L12" s="46"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="44" t="s">
-        <v>149</v>
-      </c>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
-      <c r="I13" s="44"/>
-      <c r="J13" s="44"/>
-      <c r="K13" s="44"/>
-      <c r="L13" s="44"/>
+      <c r="A13" s="46" t="s">
+        <v>171</v>
+      </c>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="46"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="46"/>
+      <c r="I13" s="46"/>
+      <c r="J13" s="46"/>
+      <c r="K13" s="46"/>
+      <c r="L13" s="46"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="43" t="s">
-        <v>150</v>
-      </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
+      <c r="A14" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="B14" s="44"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3478,12 +3990,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3494,293 +4006,307 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="45" t="s">
-        <v>152</v>
-      </c>
-      <c r="B3" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="C3" s="45" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" s="45" t="s">
-        <v>155</v>
+      <c r="A3" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="C3" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="D3" s="57" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="46" t="n">
+      <c r="A4" s="58" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>157</v>
+        <v>178</v>
+      </c>
+      <c r="C4" s="59" t="s">
+        <v>179</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="46" t="n">
+      <c r="A5" s="58" t="n">
         <v>2</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="C5" s="47" t="s">
-        <v>159</v>
+        <v>178</v>
+      </c>
+      <c r="C5" s="59" t="s">
+        <v>181</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>160</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="46" t="n">
+      <c r="A6" s="58" t="n">
         <v>3</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="C6" s="47" t="s">
-        <v>161</v>
+        <v>178</v>
+      </c>
+      <c r="C6" s="59" t="s">
+        <v>183</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="46" t="n">
+      <c r="A7" s="58" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="C7" s="47" t="s">
-        <v>164</v>
+      <c r="B7" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="C7" s="59" t="s">
+        <v>186</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="46" t="n">
+      <c r="A8" s="58" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="C8" s="47" t="s">
-        <v>166</v>
+      <c r="B8" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="46" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="58" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="C9" s="47" t="s">
-        <v>168</v>
+      <c r="B9" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="59" t="s">
+        <v>190</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="46" t="n">
+      <c r="A10" s="58" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="49" t="s">
-        <v>170</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>171</v>
+      <c r="B10" s="60" t="s">
+        <v>185</v>
+      </c>
+      <c r="C10" s="59" t="s">
+        <v>192</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="46" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="58" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="49" t="s">
-        <v>170</v>
+      <c r="B11" s="61" t="s">
+        <v>194</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="58" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="61" t="s">
+        <v>194</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="46" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="49" t="s">
-        <v>170</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>174</v>
-      </c>
       <c r="D12" s="8" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46" t="n">
+      <c r="A13" s="58" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="49" t="s">
-        <v>176</v>
+      <c r="B13" s="61" t="s">
+        <v>194</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="46" t="n">
+      <c r="A14" s="58" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="49" t="s">
-        <v>176</v>
+      <c r="B14" s="61" t="s">
+        <v>200</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="46" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="58" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="49" t="s">
-        <v>176</v>
+      <c r="B15" s="61" t="s">
+        <v>200</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="46" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="58" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="49" t="s">
-        <v>176</v>
+      <c r="B16" s="61" t="s">
+        <v>200</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>183</v>
+        <v>205</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="50" t="s">
-        <v>185</v>
+        <v>206</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="58" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="61" t="s">
+        <v>200</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="52" t="s">
-        <v>187</v>
-      </c>
-      <c r="C19" s="52"/>
-      <c r="D19" s="52"/>
+      <c r="A19" s="62" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B20" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="C20" s="52"/>
-      <c r="D20" s="52"/>
+      <c r="A20" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" s="64" t="s">
+        <v>211</v>
+      </c>
+      <c r="C20" s="64"/>
+      <c r="D20" s="64"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B21" s="52" t="s">
-        <v>189</v>
-      </c>
-      <c r="C21" s="52"/>
-      <c r="D21" s="52"/>
+      <c r="A21" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B21" s="64" t="s">
+        <v>212</v>
+      </c>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B22" s="52" t="s">
-        <v>190</v>
-      </c>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
+      <c r="A22" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B22" s="64" t="s">
+        <v>213</v>
+      </c>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B23" s="52" t="s">
-        <v>191</v>
-      </c>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
+      <c r="A23" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B23" s="64" t="s">
+        <v>214</v>
+      </c>
+      <c r="C23" s="64"/>
+      <c r="D23" s="64"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B24" s="52" t="s">
-        <v>192</v>
-      </c>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
+      <c r="A24" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B24" s="64" t="s">
+        <v>215</v>
+      </c>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51" t="s">
-        <v>186</v>
-      </c>
-      <c r="B25" s="52" t="s">
-        <v>193</v>
-      </c>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
+      <c r="A25" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B25" s="64" t="s">
+        <v>216</v>
+      </c>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="63" t="s">
+        <v>210</v>
+      </c>
+      <c r="B26" s="64" t="s">
+        <v>217</v>
+      </c>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Correct refrigerant type from stated fact to derived assumption
No document in the shipment names the refrigerant. The invoices and
instructions say only "s chladicim mediem" plus tonnes CO2e per unit.
R32 was inferred from the F-gas breakdown (0,675 t CO2e / GWP 675 =
exactly 1,000 kg), which is a strong indication but not evidence.

Removes R32 from goods descriptions and headings, marks the GWP input
and the derived kg figures as unconfirmed, and adds a critical flag:
the F-gas declaration of conformity must name the gas, so the type and
charge have to be obtained from the sender before filing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014P3Ppg3YXwLjMLjTUfeWQh
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
+++ b/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="220">
   <si>
     <t xml:space="preserve">SOUHRN HS KÓDŮ / HS CODE SUMMARY</t>
   </si>
@@ -158,10 +158,10 @@
     <t xml:space="preserve">84151090</t>
   </si>
   <si>
-    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní jednotky bez obsahu chladícího média a venkovní jednotky s chladícím médiem R32, předplněné</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split-system air conditioners – indoor units (no refrigerant) and outdoor units pre-charged with R32</t>
+    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní jednotky bez obsahu chladícího média a venkovní jednotky s chladícím médiem, předplněné</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split-system air conditioners – indoor units (no refrigerant) and outdoor units pre-charged with F-gas</t>
   </si>
   <si>
     <t xml:space="preserve">FOB WAIYUN, ZHONGSHAN, CHINA</t>
@@ -179,7 +179,7 @@
     <t xml:space="preserve">Nezjištěno – ověřit v TARIC</t>
   </si>
   <si>
-    <t xml:space="preserve">Obsahuje F-plyny (R32) – viz list „F-gas“. Kontrola kvót dle nař. (EU) 2024/573 nutná.</t>
+    <t xml:space="preserve">Obsahuje F-plyny – viz list „F-gas“. Druh chladiva v dokladech NEUVEDEN. Kontrola kvót dle nař. (EU) 2024/573 nutná.</t>
   </si>
   <si>
     <t xml:space="preserve">84159000</t>
@@ -236,7 +236,7 @@
     <t xml:space="preserve">Venkovní / Outdoor</t>
   </si>
   <si>
-    <t xml:space="preserve">Venkovní klimatizační jednotky s chladícím médiem R32</t>
+    <t xml:space="preserve">Venkovní klimatizační jednotky s chladícím médiem</t>
   </si>
   <si>
     <t xml:space="preserve">STAVBA CELNÍ HODNOTY / CUSTOMS VALUE BUILD-UP</t>
@@ -278,7 +278,7 @@
     <t xml:space="preserve">+ F-gas příspěvek (FAD-1273-2026 2 117,00 EUR + FAD-1274-2026 0,00 EUR po slevě)</t>
   </si>
   <si>
-    <t xml:space="preserve">K ROZHODNUTÍ: příspěvek za kvótu HFC účtovaný prodávajícím jako podmínka prodeje zboží obsahujícího R32 (vztahuje se jen k HS 84151090). Doporučuji zahrnout do celní hodnoty; potvrdit s klientem. Pokud by se – stejně jako u zboží zdarma – dopočetl i příspěvek k FOC jednotkám (18,20 EUR), byla by částka 2 135,20 EUR.</t>
+    <t xml:space="preserve">K ROZHODNUTÍ: příspěvek za kvótu HFC účtovaný prodávajícím jako podmínka prodeje zboží obsahujícího F-plyny (vztahuje se jen k HS 84151090). Doporučuji zahrnout do celní hodnoty; potvrdit s klientem. Pokud by se – stejně jako u zboží zdarma – dopočetl i příspěvek k FOC jednotkám (18,20 EUR), byla by částka 2 135,20 EUR.</t>
   </si>
   <si>
     <t xml:space="preserve">CELNÍ HODNOTA VČETNĚ F-GAS PŘÍSPĚVKU (bez dopravného do EU)</t>
@@ -317,7 +317,7 @@
     <t xml:space="preserve">F-plyny (t CO2e)</t>
   </si>
   <si>
-    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní bez chladícího média a venkovní předplněné R32 (placené zboží)</t>
+    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní bez chladícího média a venkovní předplněné chladivem (placené zboží)</t>
   </si>
   <si>
     <t xml:space="preserve">FAD-1271-2026</t>
@@ -458,7 +458,7 @@
     <t xml:space="preserve">YDAS-025R-09M25</t>
   </si>
   <si>
-    <t xml:space="preserve">Venkovní klimatizační jednotka s chladícím médiem R32 (split)</t>
+    <t xml:space="preserve">Venkovní klimatizační jednotka s chladícím médiem, předplněná (split)</t>
   </si>
   <si>
     <t xml:space="preserve">7SP063296</t>
@@ -497,16 +497,16 @@
     <t xml:space="preserve">Pozn.: hodnoty položek převzaty přesně z faktur (u některých řádků se součin ks × jedn. cena liší o pár centů kvůli zaokrouhlení na faktuře – rozhodující je fakturovaná hodnota).</t>
   </si>
   <si>
-    <t xml:space="preserve">F-PLYNY / F-GAS – předplněná zařízení (HFC R32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zdroj: FAD-1273-2026 (F-gas k placeným jednotkám) a FAD-1274-2026 (F-gas k jednotkám zdarma, sleva -100 %). Náplň R32, GWP 675 – odvozeno z t CO2e/jednotku.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GWP R32 (AR4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vstupní hodnota / input. Kontrola: 0,675 t CO2e ÷ 675 × 1000 = přesně 1,000 kg R32 → chladivo potvrzeno jako R32.</t>
+    <t xml:space="preserve">F-PLYNY / F-GAS – zařízení předplněná fluorovaným skleníkovým plynem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zdroj: FAD-1273-2026 (F-gas k placeným jednotkám) a FAD-1274-2026 (F-gas k jednotkám zdarma, sleva -100 %). POZOR: druh chladiva NENÍ v žádném dokladu uveden. R32 je ODVOZEN z t CO2e/jednotku – nutno potvrdit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GWP – předpoklad R32 (AR4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vstupní hodnota / input – NEPOTVRZENÁ. Druh chladiva není v dokladech uveden. R32 (GWP 675 dle AR4) je pouze ODVOZEN: 0,675 ÷ 675 × 1000 = 1,000 kg a 0,351 ÷ 675 × 1000 = 0,520 kg. Sloupce I a J jsou proto ORIENTAČNÍ.</t>
   </si>
   <si>
     <t xml:space="preserve">Model</t>
@@ -521,10 +521,10 @@
     <t xml:space="preserve">t CO2e celkem</t>
   </si>
   <si>
-    <t xml:space="preserve">Náplň R32 / unit (kg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Náplň R32 celkem (kg)</t>
+    <t xml:space="preserve">Náplň chladiva / unit (kg) – odvozeno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Náplň chladiva celkem (kg) – odvozeno</t>
   </si>
   <si>
     <t xml:space="preserve">EUR / jednotka</t>
@@ -569,10 +569,16 @@
     <t xml:space="preserve">V žádném z dokladů (FAD-1271/1272/1273/1274-2026, Packing List, HBL, instrukce) NENÍ preferenční věta (prohlášení o preferenčním původu). Původ zboží je ČÍNA („MADE IN CHINA“, „Country of origin: CHINE“). S Čínou nemá EU preferenční dohodu, takže preferenční sazbu nelze uplatnit ani doložit – uplatní se STANDARDNÍ TŘETIZEMNÍ (erga omnes) CLO. Prodávající je sice francouzská firma, ale to na původ nemá vliv.</t>
   </si>
   <si>
-    <t xml:space="preserve">F-plyny (HFC R32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venkovní jednotky YDAS-*R jsou předplněny chladivem R32: celkem 106,76 t CO2e (105,85 t placené + 0,91 t FOC), tj. cca 158 kg R32. Dovoz zařízení předplněného HFC podléhá nař. (EU) 2024/573 – dovozce (KLIMATIKA) musí být registrován ve F-Gas Portálu, musí mít pokrytí kvótou/oprávněním a v celním prohlášení se uvádí odkaz na prohlášení o shodě. BEZ TOHO CELNÍ ÚŘAD ZBOŽÍ NEPROPUSTÍ. Ověřit u klienta před podáním JSD.</t>
+    <t xml:space="preserve">F-plyny (HFC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Venkovní jednotky YDAS-*R jsou předplněny F-plynem: celkem 106,76 t CO2e (105,85 t placené + 0,91 t FOC). Dovoz zařízení předplněného HFC podléhá nař. (EU) 2024/573 – dovozce (KLIMATIKA) musí být registrován ve F-Gas Portálu, musí mít pokrytí kvótou/oprávněním a v celním prohlášení se uvádí odkaz na prohlášení o shodě. BEZ TOHO CELNÍ ÚŘAD ZBOŽÍ NEPROPUSTÍ. Ověřit u klienta před podáním JSD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Druh chladiva NENÍ v dokladech uveden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V ŽÁDNÉM z podkladů (faktury FAD-1271/1272/1273/1274-2026, Packing List, HBL, INSTRUKCE) není uveden druh chladiva. Doklady uvádějí pouze „s chladícím médiem“ a přepočet na t CO2e. R32 je v tomto souboru pouze ODVOZEN z rozpisu na FAD-1273-2026 (0,675 t CO2e ÷ GWP 675 = přesně 1,000 kg; 0,351 ÷ 675 = 0,520 kg – sedí u všech čtyř modelů). Je to silná indicie, NE doklad. Prohlášení o shodě pro F-plyny musí plyn výslovně pojmenovat, proto je nutné si druh chladiva a náplň v kg vyžádat od odesílatele (nebo doložit technickým listem / štítkem jednotky) PŘED podáním JSD.</t>
   </si>
   <si>
     <t xml:space="preserve">Chybí přepravné do celní hodnoty</t>
@@ -3995,7 +4001,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -4054,7 +4060,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="58" t="n">
         <v>3</v>
       </c>
@@ -4068,26 +4074,26 @@
         <v>184</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="58" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="59" t="s">
         <v>185</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="D7" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="8" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="58" t="n">
         <v>5</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C8" s="59" t="s">
         <v>188</v>
@@ -4096,12 +4102,12 @@
         <v>189</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="58" t="n">
         <v>6</v>
       </c>
       <c r="B9" s="60" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C9" s="59" t="s">
         <v>190</v>
@@ -4110,12 +4116,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="58" t="n">
         <v>7</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C10" s="59" t="s">
         <v>192</v>
@@ -4128,28 +4134,28 @@
       <c r="A11" s="58" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="61" t="s">
+      <c r="B11" s="60" t="s">
+        <v>187</v>
+      </c>
+      <c r="C11" s="59" t="s">
         <v>194</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="58" t="n">
         <v>9</v>
       </c>
       <c r="B12" s="61" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>39</v>
+        <v>197</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4157,10 +4163,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="61" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>198</v>
+        <v>39</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>199</v>
@@ -4171,13 +4177,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="61" t="s">
+        <v>196</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="D14" s="8" t="s">
         <v>201</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4185,7 +4191,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="61" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>203</v>
@@ -4194,12 +4200,12 @@
         <v>204</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="58" t="n">
         <v>13</v>
       </c>
       <c r="B16" s="61" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>205</v>
@@ -4208,12 +4214,12 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="58" t="n">
         <v>14</v>
       </c>
       <c r="B17" s="61" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>207</v>
@@ -4222,91 +4228,105 @@
         <v>208</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="62" t="s">
+    <row r="18" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="58" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="61" t="s">
+        <v>202</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>209</v>
       </c>
+      <c r="D18" s="8" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="63" t="s">
-        <v>210</v>
-      </c>
-      <c r="B20" s="64" t="s">
+      <c r="A20" s="62" t="s">
         <v>211</v>
       </c>
-      <c r="C20" s="64"/>
-      <c r="D20" s="64"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="63" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B21" s="64" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C21" s="64"/>
       <c r="D21" s="64"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="63" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B22" s="64" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C22" s="64"/>
       <c r="D22" s="64"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="63" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B23" s="64" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C23" s="64"/>
       <c r="D23" s="64"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="63" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B24" s="64" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C24" s="64"/>
       <c r="D24" s="64"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="63" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B25" s="64" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C25" s="64"/>
       <c r="D25" s="64"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="63" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B26" s="64" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C26" s="64"/>
       <c r="D26" s="64"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="63" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" s="64" t="s">
+        <v>219</v>
+      </c>
+      <c r="C27" s="64"/>
+      <c r="D27" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B20:D20"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B27:D27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Split HS 84151090 by refrigerant content; sharpen COO note
Main table now carries one row per HS code AND refrigerant status, as
requested, replacing the merge-to-unique-HS default: indoor units
without refrigerant, outdoor units pre-charged with F-gas, and wifi
parts. Adds explicit "CHLADIVO" and t CO2e columns. Totals are
unchanged (744 pcs, 8 690,81 kg net, 55 378,93 EUR); the deviation from
the standing merge rule is documented in the notes sheet.

Declaration items follow the same logic, now five items split by HS
code, refrigerant content and paid/FOC status.

COO note rewritten: origin IS declared on the commercial invoices
(MADE IN CHINA plus "Country of origin: CHINE" on every line, 13x and
6x), and a separate note records that no standalone certificate of
origin is present and that none is required for this import.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014P3Ppg3YXwLjMLjTUfeWQh
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
+++ b/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="231">
   <si>
     <t xml:space="preserve">SOUHRN HS KÓDŮ / HS CODE SUMMARY</t>
   </si>
@@ -107,6 +107,12 @@
     <t xml:space="preserve">HS kód</t>
   </si>
   <si>
+    <t xml:space="preserve">Typ / Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHLADIVO (F-plyny)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Popis zboží (CZ)</t>
   </si>
   <si>
@@ -134,6 +140,9 @@
     <t xml:space="preserve">CELNÍ HODNOTA (EUR)</t>
   </si>
   <si>
+    <t xml:space="preserve">F-plyny (t CO2e, dle rozpisu jednotek)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Incoterm</t>
   </si>
   <si>
@@ -149,19 +158,25 @@
     <t xml:space="preserve">Antidumping</t>
   </si>
   <si>
-    <t xml:space="preserve">Poznámka / Note</t>
-  </si>
-  <si>
     <t xml:space="preserve">GROUPE AIRWELL SA (FR)</t>
   </si>
   <si>
     <t xml:space="preserve">84151090</t>
   </si>
   <si>
-    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní jednotky bez obsahu chladícího média a venkovní jednotky s chladícím médiem, předplněné</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Split-system air conditioners – indoor units (no refrigerant) and outdoor units pre-charged with F-gas</t>
+    <t xml:space="preserve">Vnitřní / Indoor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NE – bez chladiva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky typu split – VNITŘNÍ jednotky, BEZ obsahu chladícího média</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split-system air conditioners – INDOOR units, no refrigerant charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
   </si>
   <si>
     <t xml:space="preserve">FOB WAIYUN, ZHONGSHAN, CHINA</t>
@@ -179,34 +194,100 @@
     <t xml:space="preserve">Nezjištěno – ověřit v TARIC</t>
   </si>
   <si>
-    <t xml:space="preserve">Obsahuje F-plyny – viz list „F-gas“. Druh chladiva v dokladech NEUVEDEN. Kontrola kvót dle nař. (EU) 2024/573 nutná.</t>
+    <t xml:space="preserve">Venkovní / Outdoor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANO – předplněné</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky typu split – VENKOVNÍ jednotky, PŘEDPLNĚNÉ chladícím médiem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split-system air conditioners – OUTDOOR units, pre-charged with F-gas</t>
   </si>
   <si>
     <t xml:space="preserve">84159000</t>
   </si>
   <si>
+    <t xml:space="preserve">Díl / Part</t>
+  </si>
+  <si>
     <t xml:space="preserve">Wifi modul – části a součásti klimatizačních jednotek</t>
   </si>
   <si>
     <t xml:space="preserve">Wifi module – parts of air conditioning machines</t>
   </si>
   <si>
-    <t xml:space="preserve">Bez F-plynů. 1 karton, 246 ks.</t>
-  </si>
-  <si>
     <t xml:space="preserve">CELKEM / TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">DOPLŇKOVÝ ROZPAD HS 84151090 (informativně – vnitřní vs. venkovní jednotky)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hlavní tabulka je dle pravidla sloučena na unikátní HS kódy v rámci odesílatele. Tento rozpad slouží pro kontrolu F-plynů – celní hodnota ani sazba se jím nemění.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typ / Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Popis (CZ)</t>
+    <t xml:space="preserve">STAVBA CELNÍ HODNOTY / CUSTOMS VALUE BUILD-UP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fakturovaná hodnota zboží FAD-1271-2026 (Total Item Net Value)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placené zboží, EXW/FOB cena dle faktury.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Jednotky zdarma FOC (FAD-1272-2026) v hodnotě dle faktury</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sleva -100 % NEUPLATNĚNA pro celní účely – bezúplatné zboží nemá převodní hodnotu, oceňuje se dle čl. 74 UCC hodnotou stejného zboží (ceny z FAD-1271-2026 / FAD-1272-2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ FOB poplatek (manipulace/stuffing 470 EUR/kontejner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Součást ceny skutečně placené nebo která má být zaplacena.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEZISOUČET / SUBTOTAL (bez dopravného do EU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Odpovídá sloupci „CELNÍ HODNOTA“ v hlavní tabulce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Námořní přepravné, THC a pojištění do hranice EU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOPLNIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHYBÍ V PODKLADECH – dodání je FOB Waiyun a přepravné je „FREIGHT COLLECT“. Nutno doplnit z faktury dopravce (náklady až po vstup do celního území EU) – bez toho nelze celní hodnotu uzavřít.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ F-gas příspěvek (FAD-1273-2026 2 117,00 EUR + FAD-1274-2026 0,00 EUR po slevě)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K ROZHODNUTÍ: příspěvek za kvótu HFC účtovaný prodávajícím jako podmínka prodeje zboží obsahujícího F-plyny (vztahuje se jen k HS 84151090). Doporučuji zahrnout do celní hodnoty; potvrdit s klientem. Pokud by se – stejně jako u zboží zdarma – dopočetl i příspěvek k FOC jednotkám (18,20 EUR), byla by částka 2 135,20 EUR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CELNÍ HODNOTA VČETNĚ F-GAS PŘÍSPĚVKU (bez dopravného do EU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nezahrnuje námořní přepravné/pojištění do hranice EU – viz řádek výše.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NÁVRH POLOŽEK CELNÍHO PROHLÁŠENÍ / PROPOSED DECLARATION ITEMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jedno JSD, pět položek. Členěno (1) podle HS kódu, (2) podle obsahu chladiva a (3) podle toho, zda jde o zboží placené nebo zdarma (FOC) – to má jinou metodu hodnocení a jiný druh obchodu. Vše jsou údaje na úrovni položky, samostatná JSD proto nejsou nutná. Při podání dvou JSD: položky 1, 2, 5 na jedno, položky 3 a 4 na druhé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Přepravné do hranice EU (EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">← DOPLNIT z faktury dopravce (námořní přepravné + THC + pojištění do místa vstupu do EU). Rozvrhuje se poměrem hrubé hmotnosti. Do doplnění zůstává podíl u položek nulový.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pol. č.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHLADIVO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faktura</t>
   </si>
   <si>
     <t xml:space="preserve">Množství (ks)</t>
@@ -221,90 +302,6 @@
     <t xml:space="preserve">Hodnota zboží (EUR)</t>
   </si>
   <si>
-    <t xml:space="preserve">F-plyny (t CO2e, dle rozpisu jednotek)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vnitřní / Indoor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vnitřní klimatizační jednotky bez obsahu chladícího média</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venkovní / Outdoor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venkovní klimatizační jednotky s chladícím médiem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STAVBA CELNÍ HODNOTY / CUSTOMS VALUE BUILD-UP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fakturovaná hodnota zboží FAD-1271-2026 (Total Item Net Value)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Placené zboží, EXW/FOB cena dle faktury.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+ Jednotky zdarma FOC (FAD-1272-2026) v hodnotě dle faktury</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sleva -100 % NEUPLATNĚNA pro celní účely – bezúplatné zboží nemá převodní hodnotu, oceňuje se dle čl. 74 UCC hodnotou stejného zboží (ceny z FAD-1271-2026 / FAD-1272-2026).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+ FOB poplatek (manipulace/stuffing 470 EUR/kontejner)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Součást ceny skutečně placené nebo která má být zaplacena.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEZISOUČET / SUBTOTAL (bez dopravného do EU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Odpovídá sloupci „CELNÍ HODNOTA“ v hlavní tabulce.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+ Námořní přepravné, THC a pojištění do hranice EU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOPLNIT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHYBÍ V PODKLADECH – dodání je FOB Waiyun a přepravné je „FREIGHT COLLECT“. Nutno doplnit z faktury dopravce (náklady až po vstup do celního území EU) – bez toho nelze celní hodnotu uzavřít.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+ F-gas příspěvek (FAD-1273-2026 2 117,00 EUR + FAD-1274-2026 0,00 EUR po slevě)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K ROZHODNUTÍ: příspěvek za kvótu HFC účtovaný prodávajícím jako podmínka prodeje zboží obsahujícího F-plyny (vztahuje se jen k HS 84151090). Doporučuji zahrnout do celní hodnoty; potvrdit s klientem. Pokud by se – stejně jako u zboží zdarma – dopočetl i příspěvek k FOC jednotkám (18,20 EUR), byla by částka 2 135,20 EUR.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CELNÍ HODNOTA VČETNĚ F-GAS PŘÍSPĚVKU (bez dopravného do EU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nezahrnuje námořní přepravné/pojištění do hranice EU – viz řádek výše.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NÁVRH POLOŽEK CELNÍHO PROHLÁŠENÍ / PROPOSED DECLARATION ITEMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jedno JSD, tři položky. Zboží placené a zboží zdarma (FOC) musí být SAMOSTATNÉ POLOŽKY, protože mají jinou metodu hodnocení a jiný druh obchodu – nikoli však samostatná JSD. Stejné členění platí i v případě, že by se podávala dvě JSD (pak položka 1 + 3 na jedno, položka 2 na druhé).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Přepravné do hranice EU (EUR)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">← DOPLNIT z faktury dopravce (námořní přepravné + THC + pojištění do místa vstupu do EU). Rozvrhuje se poměrem hrubé hmotnosti. Do doplnění zůstává podíl u položek nulový.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pol. č.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faktura</t>
-  </si>
-  <si>
     <t xml:space="preserve">Podíl přepravného (EUR)</t>
   </si>
   <si>
@@ -317,7 +314,13 @@
     <t xml:space="preserve">F-plyny (t CO2e)</t>
   </si>
   <si>
-    <t xml:space="preserve">Klimatizační jednotky typu split – vnitřní bez chladícího média a venkovní předplněné chladivem (placené zboží)</t>
+    <t xml:space="preserve">Poznámka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky split – VNITŘNÍ, bez obsahu chladícího média (placené zboží)</t>
   </si>
   <si>
     <t xml:space="preserve">FAD-1271-2026</t>
@@ -329,7 +332,19 @@
     <t xml:space="preserve">11 – koupě/prodej</t>
   </si>
   <si>
-    <t xml:space="preserve">Klimatizační jednotky typu split – jednotky ZDARMA (FOC UNITS 1 %), 6 ks</t>
+    <t xml:space="preserve">Bez F-plynů.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky split – VENKOVNÍ, předplněné chladícím médiem (placené zboží)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Podléhá kvótě F-plynů dle nař. (EU) 2024/573.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky split – VNITŘNÍ, bez chladiva – jednotky ZDARMA (FOC UNITS 1 %)</t>
   </si>
   <si>
     <t xml:space="preserve">FAD-1272-2026</t>
@@ -341,6 +356,15 @@
     <t xml:space="preserve">3 – bez finanční protihodnoty</t>
   </si>
   <si>
+    <t xml:space="preserve">Sleva -100 % se pro celní hodnotu NEUPLATŇUJE – oceněno cenami stejného zboží.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klimatizační jednotky split – VENKOVNÍ, předplněné – jednotky ZDARMA (FOC UNITS 1 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sleva -100 % se NEUPLATŇUJE. Podléhá kvótě F-plynů.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CELKEM</t>
   </si>
   <si>
@@ -485,9 +509,6 @@
     <t xml:space="preserve">Wifi HDLS ZDAS (wifi module)</t>
   </si>
   <si>
-    <t xml:space="preserve">Díl / Part</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kontrola / Cross-check: kartony 499 ks, čistá hm. 8 690,81 kg, hrubá hm. 9 748,44 kg, 65,16 CBM = Packing List a HBL DK26070098-B.</t>
   </si>
   <si>
@@ -566,7 +587,16 @@
     <t xml:space="preserve">COO / preferenční věta</t>
   </si>
   <si>
-    <t xml:space="preserve">V žádném z dokladů (FAD-1271/1272/1273/1274-2026, Packing List, HBL, instrukce) NENÍ preferenční věta (prohlášení o preferenčním původu). Původ zboží je ČÍNA („MADE IN CHINA“, „Country of origin: CHINE“). S Čínou nemá EU preferenční dohodu, takže preferenční sazbu nelze uplatnit ani doložit – uplatní se STANDARDNÍ TŘETIZEMNÍ (erga omnes) CLO. Prodávající je sice francouzská firma, ale to na původ nemá vliv.</t>
+    <t xml:space="preserve">PREFERENČNÍ VĚTA NENÍ v žádném z dokladů. Původ zboží ALE deklarován je: „MADE IN CHINA“ v záhlaví faktur FAD-1271-2026 a FAD-1272-2026 a „Country of origin: CHINE“ u KAŽDÉ položky (13× na FAD-1271-2026, 6× na FAD-1272-2026) – původ je tedy doložen pro všech 498 jednotek i wifi moduly. S Čínou nemá EU preferenční dohodu, takže preferenční sazbu nelze uplatnit ani doložit – uplatní se STANDARDNÍ TŘETIZEMNÍ (erga omnes) CLO. Prodávající je francouzská firma, na původ zboží to však nemá vliv.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STŘEDNÍ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COO – samostatné osvědčení o původu chybí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mezi podklady NENÍ samostatné osvědčení o původu (Certificate of Origin). Pro dovoz z Číny do volného oběhu se nevyžaduje – nepreferenční původ postačí deklarovat na základě údajů na faktuře, a preferenci stejně uplatnit nelze. Osvědčení by bylo potřeba pouze tehdy, pokud by je vyžadoval TARIC u konkrétního opatření (např. ochranné či antidumpingové) nebo pokud si je vyžádá klient/banka. Ověřit v TARIC při podání. Původ NENÍ uveden na Packing Listu, HBL ani na F-gas fakturách – tam se opírá o obchodní faktury.</t>
   </si>
   <si>
     <t xml:space="preserve">F-plyny (HFC)</t>
@@ -614,9 +644,6 @@
     <t xml:space="preserve">V souboru INSTRUKCE je pole „Přejete si vystavit JCD (vyclení do volného oběhu) nebo T1 (tranzitní doklad)?“ PRÁZDNÉ, stejně jako „ADRESA VYCLENÍ (V PŘÍPADĚ T1)“ a kontakt na ní. Nutno doptat u klienta před zahájením.</t>
   </si>
   <si>
-    <t xml:space="preserve">STŘEDNÍ</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sazba cla</t>
   </si>
   <si>
@@ -626,6 +653,12 @@
     <t xml:space="preserve">Klimatizační jednotky ani jejich díly (kap. 8415) nejsou v příloze I nařízení o CBAM (cement, železo a ocel, hliník, hnojiva, elektřina, vodík). CBAM se na tuto zásilku NEVZTAHUJE.</t>
   </si>
   <si>
+    <t xml:space="preserve">Členění řádků – odchylka od výchozího pravidla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Na žádost je HS 84151090 rozdělen na DVA řádky podle obsahu chladiva – vnitřní jednotky bez chladícího média a venkovní jednotky předplněné F-plynem – místo standardního sloučení na jeden unikátní HS kód v rámci odesílatele. Důvod je věcný: kvótě, prohlášení o shodě a kontrole F-plynů podléhají jen venkovní jednotky, takže je nutné je vykázat odděleně. Na sazební zařazení, celní hodnotu ani clo to nemá vliv – součty zůstávají shodné (744 ks, 8 690,81 kg netto, 55 378,93 EUR).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Odesílatel – jediný</t>
   </si>
   <si>
@@ -668,7 +701,7 @@
     <t xml:space="preserve">HBL DK26070098-B (DK26070098CNWAYCZMNKFD) – TR KLIMATIKA</t>
   </si>
   <si>
-    <t xml:space="preserve">Faktura FAD-1271-2026 ze dne 03/07/2026 – placené zboží, 54 797,19 EUR</t>
+    <t xml:space="preserve">Faktura FAD-1271-2026 ze dne 03/07/2026 – placené zboží, 54 797,19 EUR (obsahuje deklaraci původu u každé položky)</t>
   </si>
   <si>
     <t xml:space="preserve">Faktura FAD-1272-2026 – jednotky zdarma (FOC UNITS 1%), 581,74 EUR před slevou -100 %</t>
@@ -771,7 +804,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF006100"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -779,7 +812,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C0006"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -827,14 +860,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFFE699"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
     <fill>
@@ -899,7 +932,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -940,6 +973,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -952,12 +989,20 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -976,76 +1021,76 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1060,22 +1105,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1084,7 +1113,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1140,11 +1169,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1412,25 +1441,27 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1453,6 +1484,8 @@
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -1475,6 +1508,8 @@
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -1497,6 +1532,8 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -1519,6 +1556,8 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -1541,6 +1580,8 @@
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
@@ -1563,6 +1604,8 @@
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
@@ -1585,6 +1628,8 @@
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -1607,6 +1652,8 @@
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
@@ -1629,6 +1676,8 @@
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
@@ -1651,6 +1700,8 @@
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -1673,6 +1724,8 @@
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
@@ -1695,6 +1748,8 @@
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
@@ -1717,6 +1772,8 @@
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
@@ -1781,531 +1838,503 @@
       <c r="Q17" s="7" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="R17" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="S17" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C18" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G18" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$G$5:$G$17,$B18,'Line items'!$F$5:$F$17,$C18)</f>
+        <v>250</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$G$5:$G$17,$B18,'Line items'!$F$5:$F$17,$C18)</f>
+        <v>2383.55</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$G$5:$G$17,$B18,'Line items'!$F$5:$F$17,$C18)</f>
+        <v>2836.44</v>
+      </c>
+      <c r="J18" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,$B18,'Line items'!$F$5:$F$17,$C18)</f>
+        <v>18647.19</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,$B18,'Line items'!$F$5:$F$17,$C18)</f>
+        <v>286.02</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <f aca="false">ROUND($C$15*J18/'Line items'!$P$18,2)</f>
+        <v>161.32</v>
+      </c>
+      <c r="M18" s="13" t="n">
+        <f aca="false">J18+K18+L18</f>
+        <v>19094.53</v>
+      </c>
+      <c r="N18" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="O18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="P18" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q18" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="R18" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="S18" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="B19" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$G$5:$G$17,$B18)</f>
-        <v>498</v>
-      </c>
-      <c r="F18" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$G$5:$G$17,$B18)</f>
-        <v>8686.81</v>
-      </c>
-      <c r="G18" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$G$5:$G$17,$B18)</f>
-        <v>9743.84</v>
-      </c>
-      <c r="H18" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,$B18)</f>
-        <v>52260.79</v>
-      </c>
-      <c r="I18" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,$B18)</f>
-        <v>581.74</v>
-      </c>
-      <c r="J18" s="11" t="n">
-        <f aca="false">ROUND($C$15*H18/'Line items'!$P$18,2)</f>
-        <v>452.12</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <f aca="false">H18+I18+J18</f>
-        <v>53294.65</v>
-      </c>
-      <c r="L18" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M18" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="N18" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="O18" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="P18" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q18" s="8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>52</v>
-      </c>
       <c r="C19" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$G$5:$G$17,$B19)</f>
-        <v>246</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$G$5:$G$17,$B19)</f>
-        <v>4</v>
+        <v>56</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="G19" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$G$5:$G$17,$B19)</f>
-        <v>4.6</v>
-      </c>
-      <c r="H19" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,$B19)</f>
-        <v>2066.4</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,$B19)</f>
-        <v>0</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <f aca="false">ROUND($C$15*H19/'Line items'!$P$18,2)</f>
-        <v>17.88</v>
+        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$G$5:$G$17,$B19,'Line items'!$F$5:$F$17,$C19)</f>
+        <v>248</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$G$5:$G$17,$B19,'Line items'!$F$5:$F$17,$C19)</f>
+        <v>6303.26</v>
+      </c>
+      <c r="I19" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$G$5:$G$17,$B19,'Line items'!$F$5:$F$17,$C19)</f>
+        <v>6907.4</v>
+      </c>
+      <c r="J19" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,$B19,'Line items'!$F$5:$F$17,$C19)</f>
+        <v>33613.6</v>
       </c>
       <c r="K19" s="12" t="n">
-        <f aca="false">H19+I19+J19</f>
-        <v>2084.28</v>
-      </c>
-      <c r="L19" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M19" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="N19" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="O19" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="P19" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q19" s="8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="16" t="n">
-        <f aca="false">SUM(E18:E19)</f>
-        <v>744</v>
-      </c>
-      <c r="F20" s="17" t="n">
-        <f aca="false">SUM(F18:F19)</f>
-        <v>8690.81</v>
-      </c>
-      <c r="G20" s="17" t="n">
-        <f aca="false">SUM(G18:G19)</f>
-        <v>9748.44</v>
-      </c>
-      <c r="H20" s="17" t="n">
-        <f aca="false">SUM(H18:H19)</f>
-        <v>54327.19</v>
-      </c>
-      <c r="I20" s="17" t="n">
-        <f aca="false">SUM(I18:I19)</f>
-        <v>581.74</v>
-      </c>
-      <c r="J20" s="17" t="n">
-        <f aca="false">SUM(J18:J19)</f>
-        <v>470</v>
-      </c>
-      <c r="K20" s="17" t="n">
-        <f aca="false">SUM(K18:K19)</f>
-        <v>55378.93</v>
-      </c>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="18"/>
-      <c r="P22" s="18"/>
-      <c r="Q22" s="18"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="19"/>
-    </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="B24" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="E24" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="F24" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="G24" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="H24" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="D25" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$F$5:$F$17,$A25)</f>
-        <v>250</v>
-      </c>
-      <c r="E25" s="21" t="n">
-        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$F$5:$F$17,$A25)</f>
-        <v>2383.55</v>
-      </c>
-      <c r="F25" s="21" t="n">
-        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$F$5:$F$17,$A25)</f>
-        <v>2836.44</v>
-      </c>
-      <c r="G25" s="21" t="n">
-        <f aca="false">SUMIFS('Line items'!$R$5:$R$17,'Line items'!$F$5:$F$17,$A25)</f>
-        <v>18933.21</v>
-      </c>
-      <c r="H25" s="22" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="D26" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$F$5:$F$17,$A26)</f>
-        <v>248</v>
-      </c>
-      <c r="E26" s="21" t="n">
-        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$F$5:$F$17,$A26)</f>
-        <v>6303.26</v>
-      </c>
-      <c r="F26" s="21" t="n">
-        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$F$5:$F$17,$A26)</f>
-        <v>6907.4</v>
-      </c>
-      <c r="G26" s="21" t="n">
-        <f aca="false">SUMIFS('Line items'!$R$5:$R$17,'Line items'!$F$5:$F$17,$A26)</f>
-        <v>33909.32</v>
-      </c>
-      <c r="H26" s="22" t="n">
+        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,$B19,'Line items'!$F$5:$F$17,$C19)</f>
+        <v>295.72</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <f aca="false">ROUND($C$15*J19/'Line items'!$P$18,2)</f>
+        <v>290.8</v>
+      </c>
+      <c r="M19" s="13" t="n">
+        <f aca="false">J19+K19+L19</f>
+        <v>34200.12</v>
+      </c>
+      <c r="N19" s="14" t="n">
         <f aca="false">'F-gas'!$H$9</f>
         <v>106.822</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
+      <c r="O19" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="P19" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q19" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="R19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="S19" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$L$5:$L$17,'Line items'!$G$5:$G$17,$B20,'Line items'!$F$5:$F$17,$C20)</f>
+        <v>246</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$M$5:$M$17,'Line items'!$G$5:$G$17,$B20,'Line items'!$F$5:$F$17,$C20)</f>
+        <v>4</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$N$5:$N$17,'Line items'!$G$5:$G$17,$B20,'Line items'!$F$5:$F$17,$C20)</f>
+        <v>4.6</v>
+      </c>
+      <c r="J20" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,$B20,'Line items'!$F$5:$F$17,$C20)</f>
+        <v>2066.4</v>
+      </c>
+      <c r="K20" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,$B20,'Line items'!$F$5:$F$17,$C20)</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <f aca="false">ROUND($C$15*J20/'Line items'!$P$18,2)</f>
+        <v>17.88</v>
+      </c>
+      <c r="M20" s="13" t="n">
+        <f aca="false">J20+K20+L20</f>
+        <v>2084.28</v>
+      </c>
+      <c r="N20" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="O20" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="P20" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q20" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="R20" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="S20" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="19" t="n">
+        <f aca="false">SUM(G18:G20)</f>
+        <v>744</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <f aca="false">SUM(H18:H20)</f>
+        <v>8690.81</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <f aca="false">SUM(I18:I20)</f>
+        <v>9748.44</v>
+      </c>
+      <c r="J21" s="20" t="n">
+        <f aca="false">SUM(J18:J20)</f>
+        <v>54327.19</v>
+      </c>
+      <c r="K21" s="20" t="n">
+        <f aca="false">SUM(K18:K20)</f>
+        <v>581.74</v>
+      </c>
+      <c r="L21" s="20" t="n">
+        <f aca="false">SUM(L18:L20)</f>
+        <v>470</v>
+      </c>
+      <c r="M21" s="20" t="n">
+        <f aca="false">SUM(M18:M20)</f>
+        <v>55378.93</v>
+      </c>
+      <c r="N21" s="18"/>
+      <c r="O21" s="18"/>
+      <c r="P21" s="18"/>
+      <c r="Q21" s="18"/>
+      <c r="R21" s="18"/>
+      <c r="S21" s="18"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="21"/>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="21"/>
+      <c r="S23" s="21"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="23" t="n">
+        <f aca="false">J21</f>
+        <v>54327.19</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24"/>
+      <c r="N24" s="24"/>
+      <c r="O24" s="24"/>
+      <c r="P24" s="24"/>
+      <c r="Q24" s="24"/>
+      <c r="R24" s="24"/>
+      <c r="S24" s="24"/>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="23" t="n">
+        <f aca="false">K21</f>
+        <v>581.74</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="I25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="K25" s="24"/>
+      <c r="L25" s="24"/>
+      <c r="M25" s="24"/>
+      <c r="N25" s="24"/>
+      <c r="O25" s="24"/>
+      <c r="P25" s="24"/>
+      <c r="Q25" s="24"/>
+      <c r="R25" s="24"/>
+      <c r="S25" s="24"/>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="23" t="n">
+        <f aca="false">L21</f>
+        <v>470</v>
+      </c>
+      <c r="H26" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="18"/>
-      <c r="P28" s="18"/>
-      <c r="Q28" s="18"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="K26" s="24"/>
+      <c r="L26" s="24"/>
+      <c r="M26" s="24"/>
+      <c r="N26" s="24"/>
+      <c r="O26" s="24"/>
+      <c r="P26" s="24"/>
+      <c r="Q26" s="24"/>
+      <c r="R26" s="24"/>
+      <c r="S26" s="24"/>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="20" t="n">
+        <f aca="false">M21</f>
+        <v>55378.93</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="25"/>
+      <c r="M27" s="25"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="25"/>
+      <c r="R27" s="25"/>
+      <c r="S27" s="25"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="B28" s="26"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="H28" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="28"/>
+      <c r="L28" s="28"/>
+      <c r="M28" s="28"/>
+      <c r="N28" s="28"/>
+      <c r="O28" s="28"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="28"/>
+      <c r="R28" s="28"/>
+      <c r="S28" s="28"/>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="24" t="n">
-        <f aca="false">H20</f>
-        <v>54327.19</v>
-      </c>
-      <c r="H29" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="I29" s="25"/>
-      <c r="J29" s="25"/>
-      <c r="K29" s="25"/>
-      <c r="L29" s="25"/>
-      <c r="M29" s="25"/>
-      <c r="N29" s="25"/>
-      <c r="O29" s="25"/>
-      <c r="P29" s="25"/>
-      <c r="Q29" s="25"/>
-    </row>
-    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="24" t="n">
-        <f aca="false">I20</f>
-        <v>581.74</v>
-      </c>
-      <c r="H30" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="I30" s="25"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="25"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="25"/>
-      <c r="O30" s="25"/>
-      <c r="P30" s="25"/>
-      <c r="Q30" s="25"/>
-    </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="24" t="n">
-        <f aca="false">J20</f>
-        <v>470</v>
-      </c>
-      <c r="H31" s="25" t="s">
+      <c r="A29" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="I31" s="25"/>
-      <c r="J31" s="25"/>
-      <c r="K31" s="25"/>
-      <c r="L31" s="25"/>
-      <c r="M31" s="25"/>
-      <c r="N31" s="25"/>
-      <c r="O31" s="25"/>
-      <c r="P31" s="25"/>
-      <c r="Q31" s="25"/>
-    </row>
-    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="23" t="n">
+        <v>2117</v>
+      </c>
+      <c r="H29" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="17" t="n">
-        <f aca="false">K20</f>
-        <v>55378.93</v>
-      </c>
-      <c r="H32" s="26" t="s">
+      <c r="I29" s="24"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="24"/>
+      <c r="L29" s="24"/>
+      <c r="M29" s="24"/>
+      <c r="N29" s="24"/>
+      <c r="O29" s="24"/>
+      <c r="P29" s="24"/>
+      <c r="Q29" s="24"/>
+      <c r="R29" s="24"/>
+      <c r="S29" s="24"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="26"/>
-      <c r="P32" s="26"/>
-      <c r="Q32" s="26"/>
-    </row>
-    <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="27" t="s">
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="29" t="n">
+        <f aca="false">G27+G29</f>
+        <v>57495.93</v>
+      </c>
+      <c r="H30" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="H33" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="I33" s="29"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="29"/>
-      <c r="L33" s="29"/>
-      <c r="M33" s="29"/>
-      <c r="N33" s="29"/>
-      <c r="O33" s="29"/>
-      <c r="P33" s="29"/>
-      <c r="Q33" s="29"/>
-    </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="23"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="24" t="n">
-        <v>2117</v>
-      </c>
-      <c r="H34" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="I34" s="25"/>
-      <c r="J34" s="25"/>
-      <c r="K34" s="25"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="25"/>
-      <c r="N34" s="25"/>
-      <c r="O34" s="25"/>
-      <c r="P34" s="25"/>
-      <c r="Q34" s="25"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="30" t="n">
-        <f aca="false">G32+G34</f>
-        <v>57495.93</v>
-      </c>
-      <c r="H35" s="31" t="s">
-        <v>86</v>
-      </c>
-      <c r="I35" s="31"/>
-      <c r="J35" s="31"/>
-      <c r="K35" s="31"/>
-      <c r="L35" s="31"/>
-      <c r="M35" s="31"/>
-      <c r="N35" s="31"/>
-      <c r="O35" s="31"/>
-      <c r="P35" s="31"/>
-      <c r="Q35" s="31"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="30"/>
+      <c r="O30" s="30"/>
+      <c r="P30" s="30"/>
+      <c r="Q30" s="30"/>
+      <c r="R30" s="30"/>
+      <c r="S30" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="C3:Q3"/>
-    <mergeCell ref="C4:Q4"/>
-    <mergeCell ref="C5:Q5"/>
-    <mergeCell ref="C6:Q6"/>
-    <mergeCell ref="C7:Q7"/>
-    <mergeCell ref="C8:Q8"/>
-    <mergeCell ref="C9:Q9"/>
-    <mergeCell ref="C10:Q10"/>
-    <mergeCell ref="C11:Q11"/>
-    <mergeCell ref="C12:Q12"/>
-    <mergeCell ref="C13:Q13"/>
-    <mergeCell ref="C14:Q14"/>
-    <mergeCell ref="A22:Q22"/>
-    <mergeCell ref="A23:Q23"/>
-    <mergeCell ref="A28:Q28"/>
+  <mergeCells count="28">
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="C3:S3"/>
+    <mergeCell ref="C4:S4"/>
+    <mergeCell ref="C5:S5"/>
+    <mergeCell ref="C6:S6"/>
+    <mergeCell ref="C7:S7"/>
+    <mergeCell ref="C8:S8"/>
+    <mergeCell ref="C9:S9"/>
+    <mergeCell ref="C10:S10"/>
+    <mergeCell ref="C11:S11"/>
+    <mergeCell ref="C12:S12"/>
+    <mergeCell ref="C13:S13"/>
+    <mergeCell ref="C14:S14"/>
+    <mergeCell ref="A23:S23"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="H24:S24"/>
+    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="H25:S25"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="H26:S26"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="H27:S27"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="H28:S28"/>
     <mergeCell ref="A29:F29"/>
-    <mergeCell ref="H29:Q29"/>
+    <mergeCell ref="H29:S29"/>
     <mergeCell ref="A30:F30"/>
-    <mergeCell ref="H30:Q30"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="H31:Q31"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="H32:Q32"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="H33:Q33"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="H34:Q34"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="H35:Q35"/>
+    <mergeCell ref="H30:S30"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2322,53 +2351,56 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="32" t="s">
-        <v>87</v>
+      <c r="A1" s="31" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
+      <c r="A2" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="D4" s="33"/>
       <c r="E4" s="34" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="F4" s="34"/>
       <c r="G4" s="34"/>
@@ -2379,324 +2411,473 @@
       <c r="L4" s="34"/>
       <c r="M4" s="34"/>
       <c r="N4" s="34"/>
+      <c r="O4" s="34"/>
+      <c r="P4" s="34"/>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>27</v>
+        <v>86</v>
       </c>
       <c r="D6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J6" s="7" t="s">
+      <c r="L6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="L6" s="7" t="s">
+      <c r="N6" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="O6" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="P6" s="7" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="35" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="37" t="s">
         <v>97</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84151090")</f>
-        <v>492</v>
+      <c r="E7" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="F7" s="11" t="n">
-        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
-        <v>8597.14</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
-        <v>9641.63</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84151090")</f>
-        <v>52260.79</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <f aca="false">ROUND('HS Code Summary'!$C$15*H7/'Line items'!$P$18,2)</f>
-        <v>452.12</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <f aca="false">ROUND(IF($D$4="",0,$D$4)*G7/'Line items'!$N$18,2)</f>
+        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Vnitřní / Indoor")</f>
+        <v>246</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Vnitřní / Indoor")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>2347.42</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Vnitřní / Indoor")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>2792.91</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Vnitřní / Indoor")</f>
+        <v>18647.19</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <f aca="false">ROUND('HS Code Summary'!$C$15*I7/'Line items'!$P$18,2)</f>
+        <v>161.32</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*H7/'Line items'!$N$18,2)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="12" t="n">
-        <f aca="false">H7+I7+J7</f>
-        <v>52712.91</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>99</v>
+      <c r="L7" s="13" t="n">
+        <f aca="false">I7+J7+K7</f>
+        <v>18808.51</v>
       </c>
       <c r="M7" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="O7" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="P7" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Venkovní / Outdoor")</f>
+        <v>246</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Venkovní / Outdoor")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>6249.72</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Venkovní / Outdoor")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>6848.72</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Venkovní / Outdoor")</f>
+        <v>33613.6</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <f aca="false">ROUND('HS Code Summary'!$C$15*I8/'Line items'!$P$18,2)</f>
+        <v>290.8</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*H8/'Line items'!$N$18,2)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <f aca="false">I8+J8+K8</f>
+        <v>33904.4</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="O8" s="38" t="n">
         <f aca="false">105.85</f>
         <v>105.85</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="n">
+      <c r="P8" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$K$5:$K$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Vnitřní / Indoor")</f>
+        <v>4</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Vnitřní / Indoor")*'Line items'!$K$5:$K$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>36.13</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Vnitřní / Indoor")*'Line items'!$K$5:$K$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>43.53</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Vnitřní / Indoor")</f>
+        <v>286.02</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*H9/'Line items'!$N$18,2)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <f aca="false">I9+J9+K9</f>
+        <v>286.02</v>
+      </c>
+      <c r="M9" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="N9" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="O9" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="P9" s="42" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$K$5:$K$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Venkovní / Outdoor")</f>
         <v>2</v>
       </c>
-      <c r="B8" s="38" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="D8" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="40" t="n">
-        <f aca="false">SUMIFS('Line items'!$K$5:$K$17,'Line items'!$G$5:$G$17,"84151090")</f>
-        <v>6</v>
-      </c>
-      <c r="F8" s="41" t="n">
-        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$K$5:$K$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
-        <v>89.67</v>
-      </c>
-      <c r="G8" s="41" t="n">
-        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*'Line items'!$K$5:$K$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
-        <v>102.21</v>
-      </c>
-      <c r="H8" s="41" t="n">
-        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,"84151090")</f>
-        <v>581.74</v>
-      </c>
-      <c r="I8" s="41" t="n">
+      <c r="G10" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Venkovní / Outdoor")*'Line items'!$K$5:$K$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+        <v>53.54</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84151090")*('Line items'!$F$5:$F$17="Venkovní / Outdoor")*'Line items'!$K$5:$K$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+        <v>58.68</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$Q$5:$Q$17,'Line items'!$G$5:$G$17,"84151090",'Line items'!$F$5:$F$17,"Venkovní / Outdoor")</f>
+        <v>295.72</v>
+      </c>
+      <c r="J10" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="41" t="n">
-        <f aca="false">ROUND(IF($D$4="",0,$D$4)*G8/'Line items'!$N$18,2)</f>
+      <c r="K10" s="12" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*H10/'Line items'!$N$18,2)</f>
         <v>0</v>
       </c>
-      <c r="K8" s="42" t="n">
-        <f aca="false">H8+I8+J8</f>
-        <v>581.74</v>
-      </c>
-      <c r="L8" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="M8" s="39" t="s">
-        <v>104</v>
-      </c>
-      <c r="N8" s="43" t="n">
+      <c r="L10" s="13" t="n">
+        <f aca="false">I10+J10+K10</f>
+        <v>295.72</v>
+      </c>
+      <c r="M10" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="N10" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="O10" s="38" t="n">
         <f aca="false">0.91</f>
         <v>0.91</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84159000")</f>
+      <c r="P10" s="42" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="36" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <f aca="false">SUMIFS('Line items'!$J$5:$J$17,'Line items'!$G$5:$G$17,"84159000",'Line items'!$F$5:$F$17,"Díl / Part")</f>
         <v>246</v>
       </c>
-      <c r="F9" s="11" t="n">
-        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84159000")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
+      <c r="G11" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84159000")*('Line items'!$F$5:$F$17="Díl / Part")*'Line items'!$J$5:$J$17*'Line items'!$M$5:$M$17/'Line items'!$L$5:$L$17)</f>
         <v>4</v>
       </c>
-      <c r="G9" s="11" t="n">
-        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84159000")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
+      <c r="H11" s="12" t="n">
+        <f aca="false">SUMPRODUCT(('Line items'!$G$5:$G$17="84159000")*('Line items'!$F$5:$F$17="Díl / Part")*'Line items'!$J$5:$J$17*'Line items'!$N$5:$N$17/'Line items'!$L$5:$L$17)</f>
         <v>4.6</v>
       </c>
-      <c r="H9" s="11" t="n">
-        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84159000")</f>
+      <c r="I11" s="12" t="n">
+        <f aca="false">SUMIFS('Line items'!$P$5:$P$17,'Line items'!$G$5:$G$17,"84159000",'Line items'!$F$5:$F$17,"Díl / Part")</f>
         <v>2066.4</v>
       </c>
-      <c r="I9" s="11" t="n">
-        <f aca="false">ROUND('HS Code Summary'!$C$15*H9/'Line items'!$P$18,2)</f>
+      <c r="J11" s="12" t="n">
+        <f aca="false">ROUND('HS Code Summary'!$C$15*I11/'Line items'!$P$18,2)</f>
         <v>17.88</v>
       </c>
-      <c r="J9" s="11" t="n">
-        <f aca="false">ROUND(IF($D$4="",0,$D$4)*G9/'Line items'!$N$18,2)</f>
+      <c r="K11" s="12" t="n">
+        <f aca="false">ROUND(IF($D$4="",0,$D$4)*H11/'Line items'!$N$18,2)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="12" t="n">
-        <f aca="false">H9+I9+J9</f>
+      <c r="L11" s="13" t="n">
+        <f aca="false">I11+J11+K11</f>
         <v>2084.28</v>
       </c>
-      <c r="L9" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="M9" s="8" t="s">
+      <c r="M11" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="N9" s="21" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="16" t="n">
-        <f aca="false">SUM(E7:E9)</f>
+      <c r="N11" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="O11" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="P11" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="19" t="n">
+        <f aca="false">SUM(F7:F11)</f>
         <v>744</v>
       </c>
-      <c r="F10" s="17" t="n">
-        <f aca="false">SUM(F7:F9)</f>
+      <c r="G12" s="20" t="n">
+        <f aca="false">SUM(G7:G11)</f>
         <v>8690.81</v>
       </c>
-      <c r="G10" s="17" t="n">
-        <f aca="false">SUM(G7:G9)</f>
+      <c r="H12" s="20" t="n">
+        <f aca="false">SUM(H7:H11)</f>
         <v>9748.44</v>
       </c>
-      <c r="H10" s="17" t="n">
-        <f aca="false">SUM(H7:H9)</f>
+      <c r="I12" s="20" t="n">
+        <f aca="false">SUM(I7:I11)</f>
         <v>54908.93</v>
       </c>
-      <c r="I10" s="17" t="n">
-        <f aca="false">SUM(I7:I9)</f>
+      <c r="J12" s="20" t="n">
+        <f aca="false">SUM(J7:J11)</f>
         <v>470</v>
       </c>
-      <c r="J10" s="17" t="n">
-        <f aca="false">SUM(J7:J9)</f>
+      <c r="K12" s="20" t="n">
+        <f aca="false">SUM(K7:K11)</f>
         <v>0</v>
       </c>
-      <c r="K10" s="17" t="n">
-        <f aca="false">SUM(K7:K9)</f>
+      <c r="L12" s="20" t="n">
+        <f aca="false">SUM(L7:L11)</f>
         <v>55378.93</v>
       </c>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="15"/>
-    </row>
-    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
-        <v>106</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="44"/>
-      <c r="J12" s="44"/>
-      <c r="K12" s="44"/>
-      <c r="L12" s="44"/>
-      <c r="M12" s="44"/>
-      <c r="N12" s="44"/>
-    </row>
-    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="45" t="s">
-        <v>107</v>
-      </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="45"/>
-      <c r="I13" s="45"/>
-      <c r="J13" s="45"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="45"/>
-      <c r="M13" s="45"/>
-      <c r="N13" s="45"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44" t="s">
-        <v>108</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44"/>
-      <c r="K14" s="44"/>
-      <c r="L14" s="44"/>
-      <c r="M14" s="44"/>
-      <c r="N14" s="44"/>
+      <c r="A14" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="43"/>
+      <c r="L14" s="43"/>
+      <c r="M14" s="43"/>
+      <c r="N14" s="43"/>
+      <c r="O14" s="43"/>
+      <c r="P14" s="43"/>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="46"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="46"/>
-      <c r="I15" s="46"/>
-      <c r="J15" s="46"/>
-      <c r="K15" s="46"/>
-      <c r="L15" s="46"/>
-      <c r="M15" s="46"/>
-      <c r="N15" s="46"/>
+      <c r="A15" s="44" t="s">
+        <v>115</v>
+      </c>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="44"/>
+      <c r="M15" s="44"/>
+      <c r="N15" s="44"/>
+      <c r="O15" s="44"/>
+      <c r="P15" s="44"/>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43"/>
+      <c r="K16" s="43"/>
+      <c r="L16" s="43"/>
+      <c r="M16" s="43"/>
+      <c r="N16" s="43"/>
+      <c r="O16" s="43"/>
+      <c r="P16" s="43"/>
+    </row>
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="45"/>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="45"/>
+      <c r="G17" s="45"/>
+      <c r="H17" s="45"/>
+      <c r="I17" s="45"/>
+      <c r="J17" s="45"/>
+      <c r="K17" s="45"/>
+      <c r="L17" s="45"/>
+      <c r="M17" s="45"/>
+      <c r="N17" s="45"/>
+      <c r="O17" s="45"/>
+      <c r="P17" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="E4:N4"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A13:N13"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="E4:P4"/>
+    <mergeCell ref="A14:P14"/>
+    <mergeCell ref="A15:P15"/>
+    <mergeCell ref="A16:P16"/>
+    <mergeCell ref="A17:P17"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2736,13 +2917,13 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="32" t="s">
-        <v>110</v>
+      <c r="A1" s="31" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2750,873 +2931,873 @@
         <v>25</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>27</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>59</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>26</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>19</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G5" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G5" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I5" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I5" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="48" t="n">
+      <c r="J5" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="K5" s="48" t="n">
+      <c r="K5" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="48" t="n">
+      <c r="L5" s="47" t="n">
         <f aca="false">J5+K5</f>
         <v>25</v>
       </c>
-      <c r="M5" s="49" t="n">
+      <c r="M5" s="48" t="n">
         <v>211.25</v>
       </c>
-      <c r="N5" s="49" t="n">
+      <c r="N5" s="48" t="n">
         <v>251.25</v>
       </c>
-      <c r="O5" s="49" t="n">
+      <c r="O5" s="48" t="n">
         <v>57.6</v>
       </c>
-      <c r="P5" s="49" t="n">
+      <c r="P5" s="48" t="n">
         <v>1440</v>
       </c>
-      <c r="Q5" s="49" t="n">
+      <c r="Q5" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R5" s="49" t="n">
+      <c r="R5" s="48" t="n">
         <f aca="false">P5+Q5</f>
         <v>1440</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G6" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G6" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I6" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I6" s="47" t="n">
         <v>64</v>
       </c>
-      <c r="J6" s="48" t="n">
+      <c r="J6" s="47" t="n">
         <v>63</v>
       </c>
-      <c r="K6" s="48" t="n">
+      <c r="K6" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="48" t="n">
+      <c r="L6" s="47" t="n">
         <f aca="false">J6+K6</f>
         <v>64</v>
       </c>
-      <c r="M6" s="49" t="n">
+      <c r="M6" s="48" t="n">
         <v>629.12</v>
       </c>
-      <c r="N6" s="49" t="n">
+      <c r="N6" s="48" t="n">
         <v>750.72</v>
       </c>
-      <c r="O6" s="49" t="n">
+      <c r="O6" s="48" t="n">
         <v>63.24</v>
       </c>
-      <c r="P6" s="49" t="n">
+      <c r="P6" s="48" t="n">
         <v>3984.12</v>
       </c>
-      <c r="Q6" s="49" t="n">
+      <c r="Q6" s="48" t="n">
         <v>63.24</v>
       </c>
-      <c r="R6" s="49" t="n">
+      <c r="R6" s="48" t="n">
         <f aca="false">P6+Q6</f>
         <v>4047.36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G7" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G7" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I7" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I7" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="J7" s="48" t="n">
+      <c r="J7" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="K7" s="48" t="n">
+      <c r="K7" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="48" t="n">
+      <c r="L7" s="47" t="n">
         <f aca="false">J7+K7</f>
         <v>25</v>
       </c>
-      <c r="M7" s="49" t="n">
+      <c r="M7" s="48" t="n">
         <v>260</v>
       </c>
-      <c r="N7" s="49" t="n">
+      <c r="N7" s="48" t="n">
         <v>288.75</v>
       </c>
-      <c r="O7" s="49" t="n">
+      <c r="O7" s="48" t="n">
         <v>104.27</v>
       </c>
-      <c r="P7" s="49" t="n">
+      <c r="P7" s="48" t="n">
         <v>2606.8</v>
       </c>
-      <c r="Q7" s="49" t="n">
+      <c r="Q7" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R7" s="49" t="n">
+      <c r="R7" s="48" t="n">
         <f aca="false">P7+Q7</f>
         <v>2606.8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G8" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G8" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I8" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I8" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="48" t="n">
+      <c r="J8" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="K8" s="48" t="n">
+      <c r="K8" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="48" t="n">
+      <c r="L8" s="47" t="n">
         <f aca="false">J8+K8</f>
         <v>10</v>
       </c>
-      <c r="M8" s="49" t="n">
+      <c r="M8" s="48" t="n">
         <v>133</v>
       </c>
-      <c r="N8" s="49" t="n">
+      <c r="N8" s="48" t="n">
         <v>157</v>
       </c>
-      <c r="O8" s="49" t="n">
+      <c r="O8" s="48" t="n">
         <v>136.8</v>
       </c>
-      <c r="P8" s="49" t="n">
+      <c r="P8" s="48" t="n">
         <v>1368</v>
       </c>
-      <c r="Q8" s="49" t="n">
+      <c r="Q8" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R8" s="49" t="n">
+      <c r="R8" s="48" t="n">
         <f aca="false">P8+Q8</f>
         <v>1368</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C9" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="D9" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>126</v>
-      </c>
       <c r="F9" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G9" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G9" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I9" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I9" s="47" t="n">
         <v>26</v>
       </c>
-      <c r="J9" s="48" t="n">
+      <c r="J9" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="K9" s="48" t="n">
+      <c r="K9" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="48" t="n">
+      <c r="L9" s="47" t="n">
         <f aca="false">J9+K9</f>
         <v>26</v>
       </c>
-      <c r="M9" s="49" t="n">
+      <c r="M9" s="48" t="n">
         <v>200.72</v>
       </c>
-      <c r="N9" s="49" t="n">
+      <c r="N9" s="48" t="n">
         <v>242.32</v>
       </c>
-      <c r="O9" s="49" t="n">
+      <c r="O9" s="48" t="n">
         <v>57.08</v>
       </c>
-      <c r="P9" s="49" t="n">
+      <c r="P9" s="48" t="n">
         <v>1426.94</v>
       </c>
-      <c r="Q9" s="49" t="n">
+      <c r="Q9" s="48" t="n">
         <v>57.08</v>
       </c>
-      <c r="R9" s="49" t="n">
+      <c r="R9" s="48" t="n">
         <f aca="false">P9+Q9</f>
         <v>1484.02</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G10" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G10" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I10" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I10" s="47" t="n">
         <v>64</v>
       </c>
-      <c r="J10" s="48" t="n">
+      <c r="J10" s="47" t="n">
         <v>63</v>
       </c>
-      <c r="K10" s="48" t="n">
+      <c r="K10" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="48" t="n">
+      <c r="L10" s="47" t="n">
         <f aca="false">J10+K10</f>
         <v>64</v>
       </c>
-      <c r="M10" s="49" t="n">
+      <c r="M10" s="48" t="n">
         <v>579.84</v>
       </c>
-      <c r="N10" s="49" t="n">
+      <c r="N10" s="48" t="n">
         <v>700.16</v>
       </c>
-      <c r="O10" s="49" t="n">
+      <c r="O10" s="48" t="n">
         <v>62.21</v>
       </c>
-      <c r="P10" s="49" t="n">
+      <c r="P10" s="48" t="n">
         <v>3919.44</v>
       </c>
-      <c r="Q10" s="49" t="n">
+      <c r="Q10" s="48" t="n">
         <v>62.21</v>
       </c>
-      <c r="R10" s="49" t="n">
+      <c r="R10" s="48" t="n">
         <f aca="false">P10+Q10</f>
         <v>3981.65</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G11" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G11" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I11" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I11" s="47" t="n">
         <v>26</v>
       </c>
-      <c r="J11" s="48" t="n">
+      <c r="J11" s="47" t="n">
         <v>25</v>
       </c>
-      <c r="K11" s="48" t="n">
+      <c r="K11" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="48" t="n">
+      <c r="L11" s="47" t="n">
         <f aca="false">J11+K11</f>
         <v>26</v>
       </c>
-      <c r="M11" s="49" t="n">
+      <c r="M11" s="48" t="n">
         <v>247.52</v>
       </c>
-      <c r="N11" s="49" t="n">
+      <c r="N11" s="48" t="n">
         <v>300.04</v>
       </c>
-      <c r="O11" s="49" t="n">
+      <c r="O11" s="48" t="n">
         <v>101.36</v>
       </c>
-      <c r="P11" s="49" t="n">
+      <c r="P11" s="48" t="n">
         <v>2533.89</v>
       </c>
-      <c r="Q11" s="49" t="n">
+      <c r="Q11" s="48" t="n">
         <v>103.49</v>
       </c>
-      <c r="R11" s="49" t="n">
+      <c r="R11" s="48" t="n">
         <f aca="false">P11+Q11</f>
         <v>2637.38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" s="47" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I12" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I12" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="48" t="n">
+      <c r="J12" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="48" t="n">
+      <c r="K12" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="48" t="n">
+      <c r="L12" s="47" t="n">
         <f aca="false">J12+K12</f>
         <v>10</v>
       </c>
-      <c r="M12" s="49" t="n">
+      <c r="M12" s="48" t="n">
         <v>122.1</v>
       </c>
-      <c r="N12" s="49" t="n">
+      <c r="N12" s="48" t="n">
         <v>146.2</v>
       </c>
-      <c r="O12" s="49" t="n">
+      <c r="O12" s="48" t="n">
         <v>136.8</v>
       </c>
-      <c r="P12" s="49" t="n">
+      <c r="P12" s="48" t="n">
         <v>1368</v>
       </c>
-      <c r="Q12" s="49" t="n">
+      <c r="Q12" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R12" s="49" t="n">
+      <c r="R12" s="48" t="n">
         <f aca="false">P12+Q12</f>
         <v>1368</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="G13" s="47" t="s">
-        <v>43</v>
+        <v>56</v>
+      </c>
+      <c r="G13" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I13" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I13" s="47" t="n">
         <v>50</v>
       </c>
-      <c r="J13" s="48" t="n">
+      <c r="J13" s="47" t="n">
         <v>50</v>
       </c>
-      <c r="K13" s="48" t="n">
+      <c r="K13" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="48" t="n">
+      <c r="L13" s="47" t="n">
         <f aca="false">J13+K13</f>
         <v>50</v>
       </c>
-      <c r="M13" s="49" t="n">
+      <c r="M13" s="48" t="n">
         <v>1019</v>
       </c>
-      <c r="N13" s="49" t="n">
+      <c r="N13" s="48" t="n">
         <v>1114</v>
       </c>
-      <c r="O13" s="49" t="n">
+      <c r="O13" s="48" t="n">
         <v>109.98</v>
       </c>
-      <c r="P13" s="49" t="n">
+      <c r="P13" s="48" t="n">
         <v>5499</v>
       </c>
-      <c r="Q13" s="49" t="n">
+      <c r="Q13" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R13" s="49" t="n">
+      <c r="R13" s="48" t="n">
         <f aca="false">P13+Q13</f>
         <v>5499</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="I14" s="47" t="n">
         <v>127</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I14" s="48" t="n">
-        <v>127</v>
-      </c>
-      <c r="J14" s="48" t="n">
+      <c r="J14" s="47" t="n">
         <v>126</v>
       </c>
-      <c r="K14" s="48" t="n">
+      <c r="K14" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="48" t="n">
+      <c r="L14" s="47" t="n">
         <f aca="false">J14+K14</f>
         <v>127</v>
       </c>
-      <c r="M14" s="49" t="n">
+      <c r="M14" s="48" t="n">
         <v>2961.64</v>
       </c>
-      <c r="N14" s="49" t="n">
+      <c r="N14" s="48" t="n">
         <v>3253.74</v>
       </c>
-      <c r="O14" s="49" t="n">
+      <c r="O14" s="48" t="n">
         <v>113.1</v>
       </c>
-      <c r="P14" s="49" t="n">
+      <c r="P14" s="48" t="n">
         <v>14250.6</v>
       </c>
-      <c r="Q14" s="49" t="n">
+      <c r="Q14" s="48" t="n">
         <v>113.1</v>
       </c>
-      <c r="R14" s="49" t="n">
+      <c r="R14" s="48" t="n">
         <f aca="false">P14+Q14</f>
         <v>14363.7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="G15" s="47" t="s">
-        <v>43</v>
+        <v>56</v>
+      </c>
+      <c r="G15" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I15" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I15" s="47" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="48" t="n">
+      <c r="J15" s="47" t="n">
         <v>50</v>
       </c>
-      <c r="K15" s="48" t="n">
+      <c r="K15" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="48" t="n">
+      <c r="L15" s="47" t="n">
         <f aca="false">J15+K15</f>
         <v>51</v>
       </c>
-      <c r="M15" s="49" t="n">
+      <c r="M15" s="48" t="n">
         <v>1541.22</v>
       </c>
-      <c r="N15" s="49" t="n">
+      <c r="N15" s="48" t="n">
         <v>1686.06</v>
       </c>
-      <c r="O15" s="49" t="n">
+      <c r="O15" s="48" t="n">
         <v>182.62</v>
       </c>
-      <c r="P15" s="49" t="n">
+      <c r="P15" s="48" t="n">
         <v>9131</v>
       </c>
-      <c r="Q15" s="49" t="n">
+      <c r="Q15" s="48" t="n">
         <v>182.62</v>
       </c>
-      <c r="R15" s="49" t="n">
+      <c r="R15" s="48" t="n">
         <f aca="false">P15+Q15</f>
         <v>9313.62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="G16" s="47" t="s">
-        <v>43</v>
+        <v>56</v>
+      </c>
+      <c r="G16" s="46" t="s">
+        <v>45</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I16" s="48" t="n">
+        <v>52</v>
+      </c>
+      <c r="I16" s="47" t="n">
         <v>20</v>
       </c>
-      <c r="J16" s="48" t="n">
+      <c r="J16" s="47" t="n">
         <v>20</v>
       </c>
-      <c r="K16" s="48" t="n">
+      <c r="K16" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="48" t="n">
+      <c r="L16" s="47" t="n">
         <f aca="false">J16+K16</f>
         <v>20</v>
       </c>
-      <c r="M16" s="49" t="n">
+      <c r="M16" s="48" t="n">
         <v>781.4</v>
       </c>
-      <c r="N16" s="49" t="n">
+      <c r="N16" s="48" t="n">
         <v>853.6</v>
       </c>
-      <c r="O16" s="49" t="n">
+      <c r="O16" s="48" t="n">
         <v>236.65</v>
       </c>
-      <c r="P16" s="49" t="n">
+      <c r="P16" s="48" t="n">
         <v>4733</v>
       </c>
-      <c r="Q16" s="49" t="n">
+      <c r="Q16" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R16" s="49" t="n">
+      <c r="R16" s="48" t="n">
         <f aca="false">P16+Q16</f>
         <v>4733</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="G17" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="H17" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H17" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I17" s="48" t="n">
+      <c r="I17" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="48" t="n">
+      <c r="J17" s="47" t="n">
         <v>246</v>
       </c>
-      <c r="K17" s="48" t="n">
+      <c r="K17" s="47" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="48" t="n">
+      <c r="L17" s="47" t="n">
         <f aca="false">J17+K17</f>
         <v>246</v>
       </c>
-      <c r="M17" s="49" t="n">
+      <c r="M17" s="48" t="n">
         <v>4</v>
       </c>
-      <c r="N17" s="49" t="n">
+      <c r="N17" s="48" t="n">
         <v>4.6</v>
       </c>
-      <c r="O17" s="49" t="n">
+      <c r="O17" s="48" t="n">
         <v>8.4</v>
       </c>
-      <c r="P17" s="49" t="n">
+      <c r="P17" s="48" t="n">
         <v>2066.4</v>
       </c>
-      <c r="Q17" s="49" t="n">
+      <c r="Q17" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="R17" s="49" t="n">
+      <c r="R17" s="48" t="n">
         <f aca="false">P17+Q17</f>
         <v>2066.4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="50" t="n">
+      <c r="A18" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="49" t="n">
         <f aca="false">SUM(I5:I17)</f>
         <v>499</v>
       </c>
-      <c r="J18" s="50" t="n">
+      <c r="J18" s="49" t="n">
         <f aca="false">SUM(J5:J17)</f>
         <v>738</v>
       </c>
-      <c r="K18" s="50" t="n">
+      <c r="K18" s="49" t="n">
         <f aca="false">SUM(K5:K17)</f>
         <v>6</v>
       </c>
-      <c r="L18" s="50" t="n">
+      <c r="L18" s="49" t="n">
         <f aca="false">SUM(L5:L17)</f>
         <v>744</v>
       </c>
-      <c r="M18" s="17" t="n">
+      <c r="M18" s="20" t="n">
         <f aca="false">SUM(M5:M17)</f>
         <v>8690.81</v>
       </c>
-      <c r="N18" s="17" t="n">
+      <c r="N18" s="20" t="n">
         <f aca="false">SUM(N5:N17)</f>
         <v>9748.44</v>
       </c>
-      <c r="O18" s="15"/>
-      <c r="P18" s="17" t="n">
+      <c r="O18" s="18"/>
+      <c r="P18" s="20" t="n">
         <f aca="false">SUM(P5:P17)</f>
         <v>54327.19</v>
       </c>
-      <c r="Q18" s="17" t="n">
+      <c r="Q18" s="20" t="n">
         <f aca="false">SUM(Q5:Q17)</f>
         <v>581.74</v>
       </c>
-      <c r="R18" s="17" t="n">
+      <c r="R18" s="20" t="n">
         <f aca="false">SUM(R5:R17)</f>
         <v>54908.93</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -3651,333 +3832,333 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="32" t="s">
-        <v>157</v>
+      <c r="A1" s="31" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B3" s="51" t="n">
+        <v>166</v>
+      </c>
+      <c r="B3" s="50" t="n">
         <v>675</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="52" t="n">
+      <c r="A5" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="51" t="n">
         <v>50</v>
       </c>
-      <c r="E5" s="52" t="n">
+      <c r="E5" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="52" t="n">
+      <c r="F5" s="51" t="n">
         <f aca="false">D5+E5</f>
         <v>50</v>
       </c>
-      <c r="G5" s="53" t="n">
+      <c r="G5" s="52" t="n">
         <v>0.351</v>
       </c>
-      <c r="H5" s="53" t="n">
+      <c r="H5" s="52" t="n">
         <f aca="false">F5*G5</f>
         <v>17.55</v>
       </c>
-      <c r="I5" s="53" t="n">
+      <c r="I5" s="52" t="n">
         <f aca="false">G5/$B$3*1000</f>
         <v>0.52</v>
       </c>
-      <c r="J5" s="53" t="n">
+      <c r="J5" s="52" t="n">
         <f aca="false">F5*I5</f>
         <v>26</v>
       </c>
-      <c r="K5" s="54" t="n">
+      <c r="K5" s="53" t="n">
         <v>7.02</v>
       </c>
-      <c r="L5" s="54" t="n">
+      <c r="L5" s="53" t="n">
         <f aca="false">F5*K5</f>
         <v>351</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" s="52" t="n">
+      <c r="A6" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="51" t="n">
         <v>126</v>
       </c>
-      <c r="E6" s="52" t="n">
+      <c r="E6" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="52" t="n">
+      <c r="F6" s="51" t="n">
         <f aca="false">D6+E6</f>
         <v>127</v>
       </c>
-      <c r="G6" s="53" t="n">
+      <c r="G6" s="52" t="n">
         <v>0.385</v>
       </c>
-      <c r="H6" s="53" t="n">
+      <c r="H6" s="52" t="n">
         <f aca="false">F6*G6</f>
         <v>48.895</v>
       </c>
-      <c r="I6" s="53" t="n">
+      <c r="I6" s="52" t="n">
         <f aca="false">G6/$B$3*1000</f>
         <v>0.57037037037037</v>
       </c>
-      <c r="J6" s="53" t="n">
+      <c r="J6" s="52" t="n">
         <f aca="false">F6*I6</f>
         <v>72.437037037037</v>
       </c>
-      <c r="K6" s="54" t="n">
+      <c r="K6" s="53" t="n">
         <v>7.7</v>
       </c>
-      <c r="L6" s="54" t="n">
+      <c r="L6" s="53" t="n">
         <f aca="false">F6*K6</f>
         <v>977.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="52" t="n">
+      <c r="A7" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="51" t="n">
         <v>50</v>
       </c>
-      <c r="E7" s="52" t="n">
+      <c r="E7" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="52" t="n">
+      <c r="F7" s="51" t="n">
         <f aca="false">D7+E7</f>
         <v>51</v>
       </c>
-      <c r="G7" s="53" t="n">
+      <c r="G7" s="52" t="n">
         <v>0.527</v>
       </c>
-      <c r="H7" s="53" t="n">
+      <c r="H7" s="52" t="n">
         <f aca="false">F7*G7</f>
         <v>26.877</v>
       </c>
-      <c r="I7" s="53" t="n">
+      <c r="I7" s="52" t="n">
         <f aca="false">G7/$B$3*1000</f>
         <v>0.780740740740741</v>
       </c>
-      <c r="J7" s="53" t="n">
+      <c r="J7" s="52" t="n">
         <f aca="false">F7*I7</f>
         <v>39.8177777777778</v>
       </c>
-      <c r="K7" s="54" t="n">
+      <c r="K7" s="53" t="n">
         <v>10.53</v>
       </c>
-      <c r="L7" s="54" t="n">
+      <c r="L7" s="53" t="n">
         <f aca="false">F7*K7</f>
         <v>537.03</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="52" t="n">
+      <c r="A8" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="51" t="n">
         <v>20</v>
       </c>
-      <c r="E8" s="52" t="n">
+      <c r="E8" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="52" t="n">
+      <c r="F8" s="51" t="n">
         <f aca="false">D8+E8</f>
         <v>20</v>
       </c>
-      <c r="G8" s="53" t="n">
+      <c r="G8" s="52" t="n">
         <v>0.675</v>
       </c>
-      <c r="H8" s="53" t="n">
+      <c r="H8" s="52" t="n">
         <f aca="false">F8*G8</f>
         <v>13.5</v>
       </c>
-      <c r="I8" s="53" t="n">
+      <c r="I8" s="52" t="n">
         <f aca="false">G8/$B$3*1000</f>
         <v>1</v>
       </c>
-      <c r="J8" s="53" t="n">
+      <c r="J8" s="52" t="n">
         <f aca="false">F8*I8</f>
         <v>20</v>
       </c>
-      <c r="K8" s="54" t="n">
+      <c r="K8" s="53" t="n">
         <v>13.5</v>
       </c>
-      <c r="L8" s="54" t="n">
+      <c r="L8" s="53" t="n">
         <f aca="false">F8*K8</f>
         <v>270</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16" t="n">
+      <c r="A9" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19" t="n">
         <f aca="false">SUM(D5:D8)</f>
         <v>246</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="19" t="n">
         <f aca="false">SUM(E5:E8)</f>
         <v>2</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="19" t="n">
         <f aca="false">SUM(F5:F8)</f>
         <v>248</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="55" t="n">
+      <c r="G9" s="18"/>
+      <c r="H9" s="54" t="n">
         <f aca="false">SUM(H5:H8)</f>
         <v>106.822</v>
       </c>
-      <c r="I9" s="15"/>
-      <c r="J9" s="55" t="n">
+      <c r="I9" s="18"/>
+      <c r="J9" s="54" t="n">
         <f aca="false">SUM(J5:J8)</f>
         <v>158.254814814815</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="56" t="n">
+      <c r="K9" s="18"/>
+      <c r="L9" s="55" t="n">
         <f aca="false">SUM(L5:L8)</f>
         <v>2135.93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44" t="s">
-        <v>169</v>
-      </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
-      <c r="I11" s="44"/>
-      <c r="J11" s="44"/>
-      <c r="K11" s="44"/>
-      <c r="L11" s="44"/>
+      <c r="A11" s="43" t="s">
+        <v>176</v>
+      </c>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="46"/>
-      <c r="K12" s="46"/>
-      <c r="L12" s="46"/>
+      <c r="A12" s="45" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="45"/>
+      <c r="G12" s="45"/>
+      <c r="H12" s="45"/>
+      <c r="I12" s="45"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="45"/>
+      <c r="L12" s="45"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="46" t="s">
-        <v>171</v>
-      </c>
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="46"/>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46"/>
-      <c r="H13" s="46"/>
-      <c r="I13" s="46"/>
-      <c r="J13" s="46"/>
-      <c r="K13" s="46"/>
-      <c r="L13" s="46"/>
+      <c r="A13" s="45" t="s">
+        <v>178</v>
+      </c>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="45"/>
+      <c r="L13" s="45"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44" t="s">
-        <v>172</v>
-      </c>
-      <c r="B14" s="44"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-      <c r="H14" s="44"/>
-      <c r="I14" s="44"/>
-      <c r="J14" s="44"/>
-      <c r="K14" s="44"/>
-      <c r="L14" s="44"/>
+      <c r="A14" s="43" t="s">
+        <v>179</v>
+      </c>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="43"/>
+      <c r="L14" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4001,7 +4182,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -4012,321 +4193,349 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="57" t="s">
-        <v>174</v>
-      </c>
-      <c r="B3" s="57" t="s">
-        <v>175</v>
-      </c>
-      <c r="C3" s="57" t="s">
-        <v>176</v>
-      </c>
-      <c r="D3" s="57" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="58" t="n">
+      <c r="A3" s="56" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3" s="56" t="s">
+        <v>182</v>
+      </c>
+      <c r="C3" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="D3" s="56" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C4" s="59" t="s">
-        <v>179</v>
+      <c r="B4" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" s="58" t="s">
+        <v>186</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="58" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C5" s="59" t="s">
-        <v>181</v>
+      <c r="B5" s="59" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>189</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="58" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="57" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C6" s="59" t="s">
-        <v>183</v>
+      <c r="B6" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6" s="58" t="s">
+        <v>191</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="58" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="57" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C7" s="59" t="s">
+      <c r="B7" s="15" t="s">
         <v>185</v>
       </c>
+      <c r="C7" s="58" t="s">
+        <v>193</v>
+      </c>
       <c r="D7" s="8" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="58" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="57" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="C8" s="59" t="s">
+      <c r="B8" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="C8" s="58" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" s="58" t="s">
+        <v>198</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="57" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="60" t="s">
+        <v>197</v>
+      </c>
+      <c r="C10" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="57" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="60" t="s">
+        <v>197</v>
+      </c>
+      <c r="C11" s="58" t="s">
+        <v>202</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="57" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="60" t="s">
+        <v>197</v>
+      </c>
+      <c r="C12" s="58" t="s">
+        <v>204</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="57" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="59" t="s">
         <v>188</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="58" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="C9" s="59" t="s">
-        <v>190</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="58" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="C10" s="59" t="s">
-        <v>192</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="58" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="C11" s="59" t="s">
-        <v>194</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="58" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="61" t="s">
-        <v>196</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="58" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="61" t="s">
-        <v>196</v>
-      </c>
       <c r="C13" s="8" t="s">
-        <v>39</v>
+        <v>206</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="58" t="n">
+      <c r="A14" s="57" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="61" t="s">
-        <v>196</v>
+      <c r="B14" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>200</v>
+        <v>42</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="58" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="57" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="61" t="s">
-        <v>202</v>
+      <c r="B15" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="58" t="n">
+      <c r="A16" s="57" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="61" t="s">
-        <v>202</v>
+      <c r="B16" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="58" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="57" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="61" t="s">
-        <v>202</v>
+      <c r="B17" s="59" t="s">
+        <v>213</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="58" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="57" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="61" t="s">
-        <v>202</v>
+      <c r="B18" s="59" t="s">
+        <v>213</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="62" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B21" s="64" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="57" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="59" t="s">
         <v>213</v>
       </c>
-      <c r="C21" s="64"/>
-      <c r="D21" s="64"/>
+      <c r="C19" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="57" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="59" t="s">
+        <v>213</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B22" s="64" t="s">
-        <v>214</v>
-      </c>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
+      <c r="A22" s="61" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B23" s="64" t="s">
-        <v>215</v>
-      </c>
-      <c r="C23" s="64"/>
-      <c r="D23" s="64"/>
+      <c r="A23" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B23" s="63" t="s">
+        <v>224</v>
+      </c>
+      <c r="C23" s="63"/>
+      <c r="D23" s="63"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B24" s="64" t="s">
-        <v>216</v>
-      </c>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
+      <c r="A24" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B24" s="63" t="s">
+        <v>225</v>
+      </c>
+      <c r="C24" s="63"/>
+      <c r="D24" s="63"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B25" s="64" t="s">
-        <v>217</v>
-      </c>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
+      <c r="A25" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B25" s="63" t="s">
+        <v>226</v>
+      </c>
+      <c r="C25" s="63"/>
+      <c r="D25" s="63"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B26" s="64" t="s">
-        <v>218</v>
-      </c>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
+      <c r="A26" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B26" s="63" t="s">
+        <v>227</v>
+      </c>
+      <c r="C26" s="63"/>
+      <c r="D26" s="63"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="63" t="s">
-        <v>212</v>
-      </c>
-      <c r="B27" s="64" t="s">
-        <v>219</v>
-      </c>
-      <c r="C27" s="64"/>
-      <c r="D27" s="64"/>
+      <c r="A27" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B27" s="63" t="s">
+        <v>228</v>
+      </c>
+      <c r="C27" s="63"/>
+      <c r="D27" s="63"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B28" s="63" t="s">
+        <v>229</v>
+      </c>
+      <c r="C28" s="63"/>
+      <c r="D28" s="63"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B29" s="63" t="s">
+        <v>230</v>
+      </c>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="B26:D26"/>
     <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add dedicated FOC sheet for FAD-1272-2026 and FAD-1274-2026
New "FOC" sheet breaks the free-of-charge part of the shipment down
line by line: six goods lines from FAD-1272-2026 with net and gross
weight apportioned from the packing list, then FAD-1274-2026 shown
separately as a service with no weight, then the combined totals.

  Net weight   89,67 kg
  Gross weight 102,21 kg
  Value        581,74 + 18,20 = 599,94 EUR

Customs value build-up now adds 2 135,20 EUR of F-gas contribution
(paid plus FOC) rather than 2 117,00, applying the same identical-goods
logic to the FOC units as to the FOC goods themselves.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014P3Ppg3YXwLjMLjTUfeWQh
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
+++ b/output/HS_Code_Summary_Klimatika_DK26070098B.xlsx
@@ -10,9 +10,10 @@
   <sheets>
     <sheet name="HS Code Summary" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="JSD položky" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Line items" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="F-gas" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Kontroly &amp; poznámky" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="FOC" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Line items" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="F-gas" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Kontroly &amp; poznámky" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="263">
   <si>
     <t xml:space="preserve">SOUHRN HS KÓDŮ / HS CODE SUMMARY</t>
   </si>
@@ -257,10 +258,10 @@
     <t xml:space="preserve">CHYBÍ V PODKLADECH – dodání je FOB Waiyun a přepravné je „FREIGHT COLLECT“. Nutno doplnit z faktury dopravce (náklady až po vstup do celního území EU) – bez toho nelze celní hodnotu uzavřít.</t>
   </si>
   <si>
-    <t xml:space="preserve">+ F-gas příspěvek (FAD-1273-2026 2 117,00 EUR + FAD-1274-2026 0,00 EUR po slevě)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K ROZHODNUTÍ: příspěvek za kvótu HFC účtovaný prodávajícím jako podmínka prodeje zboží obsahujícího F-plyny (vztahuje se jen k HS 84151090). Doporučuji zahrnout do celní hodnoty; potvrdit s klientem. Pokud by se – stejně jako u zboží zdarma – dopočetl i příspěvek k FOC jednotkám (18,20 EUR), byla by částka 2 135,20 EUR.</t>
+    <t xml:space="preserve">+ F-gas příspěvek (FAD-1273-2026 2 117,00 EUR + FAD-1274-2026 18,20 EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K ROZHODNUTÍ: příspěvek za kvótu HFC účtovaný prodávajícím jako podmínka prodeje zboží obsahujícího F-plyny (vztahuje se jen k HS 84151090). Doporučuji zahrnout do celní hodnoty; potvrdit s klientem. Zahrnut i příspěvek k FOC jednotkám (18,20 EUR) – stejná logika jako u zboží zdarma. Bez FOC složky by částka činila 2 117,00 EUR.</t>
   </si>
   <si>
     <t xml:space="preserve">CELNÍ HODNOTA VČETNĚ F-GAS PŘÍSPĚVKU (bez dopravného do EU)</t>
@@ -380,6 +381,144 @@
     <t xml:space="preserve">F-plyny se deklarují za celou zásilku dohromady (106,76 t CO2e) – oprávnění/kvóta a odkaz na prohlášení o shodě musí pokrýt položku 1 i položku 2. Při rozdělení na dvě JSD je nutné uvést na obou.</t>
   </si>
   <si>
+    <t xml:space="preserve">ZBOŽÍ ZDARMA / FREE OF CHARGE – FAD-1272-2026 + FAD-1274-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kompletní rozpis bezúplatné části zásilky. Obě faktury mají slevu -100 % a fakturovanou částku 0,00 EUR; pro celní účely se hodnota NEUPLATŇUJE jako nulová – viz čl. 74 odst. 2 písm. a) UCC (hodnota stejného zboží).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A) FAD-1272-2026 – ZBOŽÍ (6 ks, jediná část zásilky s hmotností)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Řádek faktury</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kód / Product code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hodnota (EUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP024141</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDLS-035N-09M25-BK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP063296</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YDAS-035R-09M25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP063297</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YDAS-050R-09M25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP024100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDLS-025N-09M25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP024101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDLS-035N-09M25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP024102</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HDLS-050N-09M25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CELKEM FAD-1272-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B) FAD-1274-2026 – PŘÍSPĚVEK ZA F-PLYNY (služba, BEZ hmotnosti)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Popis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vztahuje se k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">t CO2e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sazba EUR/t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FGAZ – FGAS CONTRIBUTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7SP063296 × 1 ks (0,385 t) + 7SP063297 × 1 ks (0,527 t) – obě venkovní jednotky</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C) CELKEM ZBOŽÍ ZDARMA / TOTAL FOC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Počet kusů / Quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 fyzických jednotek klimatizace (4 vnitřní + 2 venkovní).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CELKOVÁ ČISTÁ HMOTNOST / TOTAL NET WEIGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pouze zboží z FAD-1272-2026. FAD-1274-2026 je služba a hmotnost nemá.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CELKOVÁ HRUBÁ HMOTNOST / TOTAL GROSS WEIGHT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozpočteno z Packing Listu podle počtu kusů (1 karton = 1 jednotka, dělí se přesně).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hodnota zboží FAD-1272-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Před slevou -100 %.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+ Příspěvek za F-plyny FAD-1274-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CELKOVÁ HODNOTA FOC / TOTAL FOC VALUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Částka k deklaraci za bezúplatnou část zásilky (za předpokladu, že se příspěvek za F-plyny zahrnuje do celní hodnoty).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrola hmotností: 89,67 kg netto a 102,21 kg brutto z 8 690,81 / 9 748,44 kg celé zásilky – zbytek (8 601,14 / 9 646,23 kg) připadá na placené zboží z FAD-1271-2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAD-1274-2026 NEMÁ hmotnost – jde o příspěvek za kvótu F-plynů (služba, reverse charge), nikoli o zboží. Do hrubé ani čisté hmotnosti se nezapočítává.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozpis na FAD-1274-2026 po jednotkách dává 0,912 t CO2e / 18,23 EUR, faktura účtuje 0,91 t / 18,20 EUR. Použita fakturovaná částka 18,20 EUR, takže celkem 581,74 + 18,20 = 599,94 EUR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jednotky zdarma jsou v Packing Listu i na HBL započteny v celkových 499 kartonech a 9 748,44 kg – fyzicky jsou součástí téhož kontejneru MRSU2515573.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ROZPIS POLOŽEK / LINE ITEM DETAIL</t>
   </si>
   <si>
@@ -389,9 +528,6 @@
     <t xml:space="preserve">Faktura / Invoice</t>
   </si>
   <si>
-    <t xml:space="preserve">Kód / Product code</t>
-  </si>
-  <si>
     <t xml:space="preserve">Model (EN)</t>
   </si>
   <si>
@@ -434,12 +570,6 @@
     <t xml:space="preserve">FAD-1271-2026 + FAD-1272-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">7SP024141</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDLS-035N-09M25-BK</t>
-  </si>
-  <si>
     <t xml:space="preserve">7SP024142</t>
   </si>
   <si>
@@ -452,24 +582,6 @@
     <t xml:space="preserve">HDLS-070N-09M25-BK</t>
   </si>
   <si>
-    <t xml:space="preserve">7SP024100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDLS-025N-09M25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7SP024101</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDLS-035N-09M25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7SP024102</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HDLS-050N-09M25</t>
-  </si>
-  <si>
     <t xml:space="preserve">7SP024103</t>
   </si>
   <si>
@@ -485,18 +597,6 @@
     <t xml:space="preserve">Venkovní klimatizační jednotka s chladícím médiem, předplněná (split)</t>
   </si>
   <si>
-    <t xml:space="preserve">7SP063296</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YDAS-035R-09M25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7SP063297</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YDAS-050R-09M25</t>
-  </si>
-  <si>
     <t xml:space="preserve">7SP063298</t>
   </si>
   <si>
@@ -528,9 +628,6 @@
   </si>
   <si>
     <t xml:space="preserve">Vstupní hodnota / input – NEPOTVRZENÁ. Druh chladiva není v dokladech uveden. R32 (GWP 675 dle AR4) je pouze ODVOZEN: 0,675 ÷ 675 × 1000 = 1,000 kg a 0,351 ÷ 675 × 1000 = 0,520 kg. Sloupce I a J jsou proto ORIENTAČNÍ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model</t>
   </si>
   <si>
     <t xml:space="preserve">Množství FOC (ks)</t>
@@ -729,7 +826,7 @@
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -813,6 +910,13 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -932,7 +1036,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="75">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1118,6 +1222,54 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1129,11 +1281,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1173,7 +1321,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2260,7 +2408,7 @@
       <c r="E29" s="22"/>
       <c r="F29" s="22"/>
       <c r="G29" s="23" t="n">
-        <v>2117</v>
+        <v>2135.2</v>
       </c>
       <c r="H29" s="24" t="s">
         <v>78</v>
@@ -2288,7 +2436,7 @@
       <c r="F30" s="18"/>
       <c r="G30" s="29" t="n">
         <f aca="false">G27+G29</f>
-        <v>57495.93</v>
+        <v>57514.13</v>
       </c>
       <c r="H30" s="30" t="s">
         <v>80</v>
@@ -2894,6 +3042,626 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J30"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="31" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+    </row>
+    <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>126</v>
+      </c>
+      <c r="C6" s="46" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="47" t="n">
+        <f aca="false">'Line items'!$K$6</f>
+        <v>1</v>
+      </c>
+      <c r="H6" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$M$6/'Line items'!$L$6*G6,2)</f>
+        <v>9.83</v>
+      </c>
+      <c r="I6" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$N$6/'Line items'!$L$6*G6,2)</f>
+        <v>11.73</v>
+      </c>
+      <c r="J6" s="48" t="n">
+        <f aca="false">'Line items'!$Q$6</f>
+        <v>63.24</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="B7" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="47" t="n">
+        <f aca="false">'Line items'!$K$14</f>
+        <v>1</v>
+      </c>
+      <c r="H7" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$M$14/'Line items'!$L$14*G7,2)</f>
+        <v>23.32</v>
+      </c>
+      <c r="I7" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$N$14/'Line items'!$L$14*G7,2)</f>
+        <v>25.62</v>
+      </c>
+      <c r="J7" s="48" t="n">
+        <f aca="false">'Line items'!$Q$14</f>
+        <v>113.1</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="47" t="n">
+        <f aca="false">'Line items'!$K$15</f>
+        <v>1</v>
+      </c>
+      <c r="H8" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$M$15/'Line items'!$L$15*G8,2)</f>
+        <v>30.22</v>
+      </c>
+      <c r="I8" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$N$15/'Line items'!$L$15*G8,2)</f>
+        <v>33.06</v>
+      </c>
+      <c r="J8" s="48" t="n">
+        <f aca="false">'Line items'!$Q$15</f>
+        <v>182.62</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="35" t="n">
+        <v>40</v>
+      </c>
+      <c r="B9" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="47" t="n">
+        <f aca="false">'Line items'!$K$9</f>
+        <v>1</v>
+      </c>
+      <c r="H9" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$M$9/'Line items'!$L$9*G9,2)</f>
+        <v>7.72</v>
+      </c>
+      <c r="I9" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$N$9/'Line items'!$L$9*G9,2)</f>
+        <v>9.32</v>
+      </c>
+      <c r="J9" s="48" t="n">
+        <f aca="false">'Line items'!$Q$9</f>
+        <v>57.08</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="35" t="n">
+        <v>50</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>135</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F10" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" s="47" t="n">
+        <f aca="false">'Line items'!$K$10</f>
+        <v>1</v>
+      </c>
+      <c r="H10" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$M$10/'Line items'!$L$10*G10,2)</f>
+        <v>9.06</v>
+      </c>
+      <c r="I10" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$N$10/'Line items'!$L$10*G10,2)</f>
+        <v>10.94</v>
+      </c>
+      <c r="J10" s="48" t="n">
+        <f aca="false">'Line items'!$Q$10</f>
+        <v>62.21</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="n">
+        <v>60</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F11" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="47" t="n">
+        <f aca="false">'Line items'!$K$11</f>
+        <v>1</v>
+      </c>
+      <c r="H11" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$M$11/'Line items'!$L$11*G11,2)</f>
+        <v>9.52</v>
+      </c>
+      <c r="I11" s="48" t="n">
+        <f aca="false">ROUND('Line items'!$N$11/'Line items'!$L$11*G11,2)</f>
+        <v>11.54</v>
+      </c>
+      <c r="J11" s="48" t="n">
+        <f aca="false">'Line items'!$Q$11</f>
+        <v>103.49</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="49" t="n">
+        <f aca="false">SUM(G6:G11)</f>
+        <v>6</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <f aca="false">SUM(H6:H11)</f>
+        <v>89.67</v>
+      </c>
+      <c r="I12" s="20" t="n">
+        <f aca="false">SUM(I6:I11)</f>
+        <v>102.21</v>
+      </c>
+      <c r="J12" s="20" t="n">
+        <f aca="false">SUM(J6:J11)</f>
+        <v>581.74</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="21"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="46" t="s">
+        <v>144</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>145</v>
+      </c>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="50" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G16" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" s="46"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="48" t="n">
+        <f aca="false">ROUND(F16*G16,2)</f>
+        <v>18.2</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="51" t="s">
+        <v>146</v>
+      </c>
+      <c r="B18" s="51"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="51"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="51"/>
+    </row>
+    <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="52" t="n">
+        <f aca="false">G12</f>
+        <v>6</v>
+      </c>
+      <c r="F19" s="53" t="s">
+        <v>148</v>
+      </c>
+      <c r="G19" s="54" t="s">
+        <v>149</v>
+      </c>
+      <c r="H19" s="54"/>
+      <c r="I19" s="54"/>
+      <c r="J19" s="54"/>
+    </row>
+    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="55" t="s">
+        <v>150</v>
+      </c>
+      <c r="B20" s="55"/>
+      <c r="C20" s="55"/>
+      <c r="D20" s="55"/>
+      <c r="E20" s="56" t="n">
+        <f aca="false">H12</f>
+        <v>89.67</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="G20" s="57" t="s">
+        <v>152</v>
+      </c>
+      <c r="H20" s="57"/>
+      <c r="I20" s="57"/>
+      <c r="J20" s="57"/>
+    </row>
+    <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="55" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" s="55"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="56" t="n">
+        <f aca="false">I12</f>
+        <v>102.21</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="G21" s="57" t="s">
+        <v>154</v>
+      </c>
+      <c r="H21" s="57"/>
+      <c r="I21" s="57"/>
+      <c r="J21" s="57"/>
+    </row>
+    <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="23" t="n">
+        <f aca="false">J12</f>
+        <v>581.74</v>
+      </c>
+      <c r="F22" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="H22" s="54"/>
+      <c r="I22" s="54"/>
+      <c r="J22" s="54"/>
+    </row>
+    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="23" t="n">
+        <f aca="false">J16</f>
+        <v>18.2</v>
+      </c>
+      <c r="F23" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54"/>
+    </row>
+    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="55" t="s">
+        <v>158</v>
+      </c>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="56" t="n">
+        <f aca="false">J16+J12</f>
+        <v>599.94</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" s="57" t="s">
+        <v>159</v>
+      </c>
+      <c r="H24" s="57"/>
+      <c r="I24" s="57"/>
+      <c r="J24" s="57"/>
+    </row>
+    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="43" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="43"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="43"/>
+      <c r="I27" s="43"/>
+      <c r="J27" s="43"/>
+    </row>
+    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="45" t="s">
+        <v>161</v>
+      </c>
+      <c r="B28" s="45"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="45"/>
+      <c r="H28" s="45"/>
+      <c r="I28" s="45"/>
+      <c r="J28" s="45"/>
+    </row>
+    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="B29" s="44"/>
+      <c r="C29" s="44"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="44"/>
+      <c r="J29" s="44"/>
+    </row>
+    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="B30" s="44"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
+      <c r="J30" s="44"/>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A30:J30"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:R22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2918,12 +3686,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>118</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>119</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2931,13 +3699,13 @@
         <v>25</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>120</v>
+        <v>166</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>122</v>
+        <v>167</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>29</v>
@@ -2955,31 +3723,31 @@
         <v>19</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>124</v>
+        <v>169</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>125</v>
+        <v>170</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>127</v>
+        <v>172</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>128</v>
+        <v>173</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>129</v>
+        <v>174</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>130</v>
+        <v>175</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>131</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2990,52 +3758,52 @@
         <v>99</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>132</v>
+        <v>177</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>133</v>
+        <v>178</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="46" t="s">
+      <c r="G5" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I5" s="47" t="n">
+      <c r="I5" s="59" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="47" t="n">
+      <c r="J5" s="59" t="n">
         <v>25</v>
       </c>
-      <c r="K5" s="47" t="n">
+      <c r="K5" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="47" t="n">
+      <c r="L5" s="59" t="n">
         <f aca="false">J5+K5</f>
         <v>25</v>
       </c>
-      <c r="M5" s="48" t="n">
+      <c r="M5" s="60" t="n">
         <v>211.25</v>
       </c>
-      <c r="N5" s="48" t="n">
+      <c r="N5" s="60" t="n">
         <v>251.25</v>
       </c>
-      <c r="O5" s="48" t="n">
+      <c r="O5" s="60" t="n">
         <v>57.6</v>
       </c>
-      <c r="P5" s="48" t="n">
+      <c r="P5" s="60" t="n">
         <v>1440</v>
       </c>
-      <c r="Q5" s="48" t="n">
+      <c r="Q5" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R5" s="48" t="n">
+      <c r="R5" s="60" t="n">
         <f aca="false">P5+Q5</f>
         <v>1440</v>
       </c>
@@ -3045,55 +3813,55 @@
         <v>44</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="46" t="s">
+      <c r="G6" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I6" s="47" t="n">
+      <c r="I6" s="59" t="n">
         <v>64</v>
       </c>
-      <c r="J6" s="47" t="n">
+      <c r="J6" s="59" t="n">
         <v>63</v>
       </c>
-      <c r="K6" s="47" t="n">
+      <c r="K6" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="47" t="n">
+      <c r="L6" s="59" t="n">
         <f aca="false">J6+K6</f>
         <v>64</v>
       </c>
-      <c r="M6" s="48" t="n">
+      <c r="M6" s="60" t="n">
         <v>629.12</v>
       </c>
-      <c r="N6" s="48" t="n">
+      <c r="N6" s="60" t="n">
         <v>750.72</v>
       </c>
-      <c r="O6" s="48" t="n">
+      <c r="O6" s="60" t="n">
         <v>63.24</v>
       </c>
-      <c r="P6" s="48" t="n">
+      <c r="P6" s="60" t="n">
         <v>3984.12</v>
       </c>
-      <c r="Q6" s="48" t="n">
+      <c r="Q6" s="60" t="n">
         <v>63.24</v>
       </c>
-      <c r="R6" s="48" t="n">
+      <c r="R6" s="60" t="n">
         <f aca="false">P6+Q6</f>
         <v>4047.36</v>
       </c>
@@ -3106,52 +3874,52 @@
         <v>99</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="46" t="s">
+      <c r="G7" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I7" s="47" t="n">
+      <c r="I7" s="59" t="n">
         <v>25</v>
       </c>
-      <c r="J7" s="47" t="n">
+      <c r="J7" s="59" t="n">
         <v>25</v>
       </c>
-      <c r="K7" s="47" t="n">
+      <c r="K7" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="47" t="n">
+      <c r="L7" s="59" t="n">
         <f aca="false">J7+K7</f>
         <v>25</v>
       </c>
-      <c r="M7" s="48" t="n">
+      <c r="M7" s="60" t="n">
         <v>260</v>
       </c>
-      <c r="N7" s="48" t="n">
+      <c r="N7" s="60" t="n">
         <v>288.75</v>
       </c>
-      <c r="O7" s="48" t="n">
+      <c r="O7" s="60" t="n">
         <v>104.27</v>
       </c>
-      <c r="P7" s="48" t="n">
+      <c r="P7" s="60" t="n">
         <v>2606.8</v>
       </c>
-      <c r="Q7" s="48" t="n">
+      <c r="Q7" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R7" s="48" t="n">
+      <c r="R7" s="60" t="n">
         <f aca="false">P7+Q7</f>
         <v>2606.8</v>
       </c>
@@ -3164,52 +3932,52 @@
         <v>99</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>141</v>
+        <v>184</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G8" s="46" t="s">
+      <c r="G8" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I8" s="47" t="n">
+      <c r="I8" s="59" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="47" t="n">
+      <c r="J8" s="59" t="n">
         <v>10</v>
       </c>
-      <c r="K8" s="47" t="n">
+      <c r="K8" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="47" t="n">
+      <c r="L8" s="59" t="n">
         <f aca="false">J8+K8</f>
         <v>10</v>
       </c>
-      <c r="M8" s="48" t="n">
+      <c r="M8" s="60" t="n">
         <v>133</v>
       </c>
-      <c r="N8" s="48" t="n">
+      <c r="N8" s="60" t="n">
         <v>157</v>
       </c>
-      <c r="O8" s="48" t="n">
+      <c r="O8" s="60" t="n">
         <v>136.8</v>
       </c>
-      <c r="P8" s="48" t="n">
+      <c r="P8" s="60" t="n">
         <v>1368</v>
       </c>
-      <c r="Q8" s="48" t="n">
+      <c r="Q8" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R8" s="48" t="n">
+      <c r="R8" s="60" t="n">
         <f aca="false">P8+Q8</f>
         <v>1368</v>
       </c>
@@ -3219,55 +3987,55 @@
         <v>44</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="46" t="s">
+      <c r="G9" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I9" s="47" t="n">
+      <c r="I9" s="59" t="n">
         <v>26</v>
       </c>
-      <c r="J9" s="47" t="n">
+      <c r="J9" s="59" t="n">
         <v>25</v>
       </c>
-      <c r="K9" s="47" t="n">
+      <c r="K9" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="47" t="n">
+      <c r="L9" s="59" t="n">
         <f aca="false">J9+K9</f>
         <v>26</v>
       </c>
-      <c r="M9" s="48" t="n">
+      <c r="M9" s="60" t="n">
         <v>200.72</v>
       </c>
-      <c r="N9" s="48" t="n">
+      <c r="N9" s="60" t="n">
         <v>242.32</v>
       </c>
-      <c r="O9" s="48" t="n">
+      <c r="O9" s="60" t="n">
         <v>57.08</v>
       </c>
-      <c r="P9" s="48" t="n">
+      <c r="P9" s="60" t="n">
         <v>1426.94</v>
       </c>
-      <c r="Q9" s="48" t="n">
+      <c r="Q9" s="60" t="n">
         <v>57.08</v>
       </c>
-      <c r="R9" s="48" t="n">
+      <c r="R9" s="60" t="n">
         <f aca="false">P9+Q9</f>
         <v>1484.02</v>
       </c>
@@ -3277,55 +4045,55 @@
         <v>44</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>145</v>
-      </c>
       <c r="E10" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="46" t="s">
+      <c r="G10" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="47" t="n">
+      <c r="I10" s="59" t="n">
         <v>64</v>
       </c>
-      <c r="J10" s="47" t="n">
+      <c r="J10" s="59" t="n">
         <v>63</v>
       </c>
-      <c r="K10" s="47" t="n">
+      <c r="K10" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="47" t="n">
+      <c r="L10" s="59" t="n">
         <f aca="false">J10+K10</f>
         <v>64</v>
       </c>
-      <c r="M10" s="48" t="n">
+      <c r="M10" s="60" t="n">
         <v>579.84</v>
       </c>
-      <c r="N10" s="48" t="n">
+      <c r="N10" s="60" t="n">
         <v>700.16</v>
       </c>
-      <c r="O10" s="48" t="n">
+      <c r="O10" s="60" t="n">
         <v>62.21</v>
       </c>
-      <c r="P10" s="48" t="n">
+      <c r="P10" s="60" t="n">
         <v>3919.44</v>
       </c>
-      <c r="Q10" s="48" t="n">
+      <c r="Q10" s="60" t="n">
         <v>62.21</v>
       </c>
-      <c r="R10" s="48" t="n">
+      <c r="R10" s="60" t="n">
         <f aca="false">P10+Q10</f>
         <v>3981.65</v>
       </c>
@@ -3335,55 +4103,55 @@
         <v>44</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G11" s="46" t="s">
+      <c r="G11" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I11" s="47" t="n">
+      <c r="I11" s="59" t="n">
         <v>26</v>
       </c>
-      <c r="J11" s="47" t="n">
+      <c r="J11" s="59" t="n">
         <v>25</v>
       </c>
-      <c r="K11" s="47" t="n">
+      <c r="K11" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="47" t="n">
+      <c r="L11" s="59" t="n">
         <f aca="false">J11+K11</f>
         <v>26</v>
       </c>
-      <c r="M11" s="48" t="n">
+      <c r="M11" s="60" t="n">
         <v>247.52</v>
       </c>
-      <c r="N11" s="48" t="n">
+      <c r="N11" s="60" t="n">
         <v>300.04</v>
       </c>
-      <c r="O11" s="48" t="n">
+      <c r="O11" s="60" t="n">
         <v>101.36</v>
       </c>
-      <c r="P11" s="48" t="n">
+      <c r="P11" s="60" t="n">
         <v>2533.89</v>
       </c>
-      <c r="Q11" s="48" t="n">
+      <c r="Q11" s="60" t="n">
         <v>103.49</v>
       </c>
-      <c r="R11" s="48" t="n">
+      <c r="R11" s="60" t="n">
         <f aca="false">P11+Q11</f>
         <v>2637.38</v>
       </c>
@@ -3396,52 +4164,52 @@
         <v>99</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>149</v>
+        <v>186</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>134</v>
+        <v>179</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="G12" s="46" t="s">
+      <c r="G12" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I12" s="47" t="n">
+      <c r="I12" s="59" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="47" t="n">
+      <c r="J12" s="59" t="n">
         <v>10</v>
       </c>
-      <c r="K12" s="47" t="n">
+      <c r="K12" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="47" t="n">
+      <c r="L12" s="59" t="n">
         <f aca="false">J12+K12</f>
         <v>10</v>
       </c>
-      <c r="M12" s="48" t="n">
+      <c r="M12" s="60" t="n">
         <v>122.1</v>
       </c>
-      <c r="N12" s="48" t="n">
+      <c r="N12" s="60" t="n">
         <v>146.2</v>
       </c>
-      <c r="O12" s="48" t="n">
+      <c r="O12" s="60" t="n">
         <v>136.8</v>
       </c>
-      <c r="P12" s="48" t="n">
+      <c r="P12" s="60" t="n">
         <v>1368</v>
       </c>
-      <c r="Q12" s="48" t="n">
+      <c r="Q12" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R12" s="48" t="n">
+      <c r="R12" s="60" t="n">
         <f aca="false">P12+Q12</f>
         <v>1368</v>
       </c>
@@ -3454,52 +4222,52 @@
         <v>99</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>151</v>
+        <v>188</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="46" t="s">
+      <c r="G13" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I13" s="47" t="n">
+      <c r="I13" s="59" t="n">
         <v>50</v>
       </c>
-      <c r="J13" s="47" t="n">
+      <c r="J13" s="59" t="n">
         <v>50</v>
       </c>
-      <c r="K13" s="47" t="n">
+      <c r="K13" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="47" t="n">
+      <c r="L13" s="59" t="n">
         <f aca="false">J13+K13</f>
         <v>50</v>
       </c>
-      <c r="M13" s="48" t="n">
+      <c r="M13" s="60" t="n">
         <v>1019</v>
       </c>
-      <c r="N13" s="48" t="n">
+      <c r="N13" s="60" t="n">
         <v>1114</v>
       </c>
-      <c r="O13" s="48" t="n">
+      <c r="O13" s="60" t="n">
         <v>109.98</v>
       </c>
-      <c r="P13" s="48" t="n">
+      <c r="P13" s="60" t="n">
         <v>5499</v>
       </c>
-      <c r="Q13" s="48" t="n">
+      <c r="Q13" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R13" s="48" t="n">
+      <c r="R13" s="60" t="n">
         <f aca="false">P13+Q13</f>
         <v>5499</v>
       </c>
@@ -3509,55 +4277,55 @@
         <v>44</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>154</v>
+        <v>129</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="G14" s="46" t="s">
+      <c r="G14" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I14" s="47" t="n">
+      <c r="I14" s="59" t="n">
         <v>127</v>
       </c>
-      <c r="J14" s="47" t="n">
+      <c r="J14" s="59" t="n">
         <v>126</v>
       </c>
-      <c r="K14" s="47" t="n">
+      <c r="K14" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="47" t="n">
+      <c r="L14" s="59" t="n">
         <f aca="false">J14+K14</f>
         <v>127</v>
       </c>
-      <c r="M14" s="48" t="n">
+      <c r="M14" s="60" t="n">
         <v>2961.64</v>
       </c>
-      <c r="N14" s="48" t="n">
+      <c r="N14" s="60" t="n">
         <v>3253.74</v>
       </c>
-      <c r="O14" s="48" t="n">
+      <c r="O14" s="60" t="n">
         <v>113.1</v>
       </c>
-      <c r="P14" s="48" t="n">
+      <c r="P14" s="60" t="n">
         <v>14250.6</v>
       </c>
-      <c r="Q14" s="48" t="n">
+      <c r="Q14" s="60" t="n">
         <v>113.1</v>
       </c>
-      <c r="R14" s="48" t="n">
+      <c r="R14" s="60" t="n">
         <f aca="false">P14+Q14</f>
         <v>14363.7</v>
       </c>
@@ -3567,55 +4335,55 @@
         <v>44</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="G15" s="46" t="s">
+      <c r="G15" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I15" s="47" t="n">
+      <c r="I15" s="59" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="47" t="n">
+      <c r="J15" s="59" t="n">
         <v>50</v>
       </c>
-      <c r="K15" s="47" t="n">
+      <c r="K15" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="47" t="n">
+      <c r="L15" s="59" t="n">
         <f aca="false">J15+K15</f>
         <v>51</v>
       </c>
-      <c r="M15" s="48" t="n">
+      <c r="M15" s="60" t="n">
         <v>1541.22</v>
       </c>
-      <c r="N15" s="48" t="n">
+      <c r="N15" s="60" t="n">
         <v>1686.06</v>
       </c>
-      <c r="O15" s="48" t="n">
+      <c r="O15" s="60" t="n">
         <v>182.62</v>
       </c>
-      <c r="P15" s="48" t="n">
+      <c r="P15" s="60" t="n">
         <v>9131</v>
       </c>
-      <c r="Q15" s="48" t="n">
+      <c r="Q15" s="60" t="n">
         <v>182.62</v>
       </c>
-      <c r="R15" s="48" t="n">
+      <c r="R15" s="60" t="n">
         <f aca="false">P15+Q15</f>
         <v>9313.62</v>
       </c>
@@ -3628,52 +4396,52 @@
         <v>99</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>157</v>
+        <v>190</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>158</v>
+        <v>191</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="G16" s="46" t="s">
+      <c r="G16" s="58" t="s">
         <v>45</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I16" s="47" t="n">
+      <c r="I16" s="59" t="n">
         <v>20</v>
       </c>
-      <c r="J16" s="47" t="n">
+      <c r="J16" s="59" t="n">
         <v>20</v>
       </c>
-      <c r="K16" s="47" t="n">
+      <c r="K16" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="47" t="n">
+      <c r="L16" s="59" t="n">
         <f aca="false">J16+K16</f>
         <v>20</v>
       </c>
-      <c r="M16" s="48" t="n">
+      <c r="M16" s="60" t="n">
         <v>781.4</v>
       </c>
-      <c r="N16" s="48" t="n">
+      <c r="N16" s="60" t="n">
         <v>853.6</v>
       </c>
-      <c r="O16" s="48" t="n">
+      <c r="O16" s="60" t="n">
         <v>236.65</v>
       </c>
-      <c r="P16" s="48" t="n">
+      <c r="P16" s="60" t="n">
         <v>4733</v>
       </c>
-      <c r="Q16" s="48" t="n">
+      <c r="Q16" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R16" s="48" t="n">
+      <c r="R16" s="60" t="n">
         <f aca="false">P16+Q16</f>
         <v>4733</v>
       </c>
@@ -3686,10 +4454,10 @@
         <v>99</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>159</v>
+        <v>192</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>160</v>
+        <v>193</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>62</v>
@@ -3697,41 +4465,41 @@
       <c r="F17" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="46" t="s">
+      <c r="G17" s="58" t="s">
         <v>60</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I17" s="47" t="n">
+      <c r="I17" s="59" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="47" t="n">
+      <c r="J17" s="59" t="n">
         <v>246</v>
       </c>
-      <c r="K17" s="47" t="n">
+      <c r="K17" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="47" t="n">
+      <c r="L17" s="59" t="n">
         <f aca="false">J17+K17</f>
         <v>246</v>
       </c>
-      <c r="M17" s="48" t="n">
+      <c r="M17" s="60" t="n">
         <v>4</v>
       </c>
-      <c r="N17" s="48" t="n">
+      <c r="N17" s="60" t="n">
         <v>4.6</v>
       </c>
-      <c r="O17" s="48" t="n">
+      <c r="O17" s="60" t="n">
         <v>8.4</v>
       </c>
-      <c r="P17" s="48" t="n">
+      <c r="P17" s="60" t="n">
         <v>2066.4</v>
       </c>
-      <c r="Q17" s="48" t="n">
+      <c r="Q17" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="R17" s="48" t="n">
+      <c r="R17" s="60" t="n">
         <f aca="false">P17+Q17</f>
         <v>2066.4</v>
       </c>
@@ -3787,17 +4555,17 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>161</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>162</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>163</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -3811,7 +4579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3833,231 +4601,231 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="31" t="s">
-        <v>164</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>165</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="B3" s="50" t="n">
+        <v>199</v>
+      </c>
+      <c r="B3" s="61" t="n">
         <v>675</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>167</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>168</v>
+        <v>123</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>123</v>
+        <v>168</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>169</v>
+        <v>201</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>125</v>
+        <v>170</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>170</v>
+        <v>202</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>171</v>
+        <v>203</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>172</v>
+        <v>204</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>173</v>
+        <v>205</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>174</v>
+        <v>206</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>175</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>151</v>
+        <v>188</v>
       </c>
       <c r="C5" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="51" t="n">
+      <c r="D5" s="62" t="n">
         <v>50</v>
       </c>
-      <c r="E5" s="51" t="n">
+      <c r="E5" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="51" t="n">
+      <c r="F5" s="62" t="n">
         <f aca="false">D5+E5</f>
         <v>50</v>
       </c>
-      <c r="G5" s="52" t="n">
+      <c r="G5" s="63" t="n">
         <v>0.351</v>
       </c>
-      <c r="H5" s="52" t="n">
+      <c r="H5" s="63" t="n">
         <f aca="false">F5*G5</f>
         <v>17.55</v>
       </c>
-      <c r="I5" s="52" t="n">
+      <c r="I5" s="63" t="n">
         <f aca="false">G5/$B$3*1000</f>
         <v>0.52</v>
       </c>
-      <c r="J5" s="52" t="n">
+      <c r="J5" s="63" t="n">
         <f aca="false">F5*I5</f>
         <v>26</v>
       </c>
-      <c r="K5" s="53" t="n">
+      <c r="K5" s="64" t="n">
         <v>7.02</v>
       </c>
-      <c r="L5" s="53" t="n">
+      <c r="L5" s="64" t="n">
         <f aca="false">F5*K5</f>
         <v>351</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>154</v>
+        <v>129</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="51" t="n">
+      <c r="D6" s="62" t="n">
         <v>126</v>
       </c>
-      <c r="E6" s="51" t="n">
+      <c r="E6" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="51" t="n">
+      <c r="F6" s="62" t="n">
         <f aca="false">D6+E6</f>
         <v>127</v>
       </c>
-      <c r="G6" s="52" t="n">
+      <c r="G6" s="63" t="n">
         <v>0.385</v>
       </c>
-      <c r="H6" s="52" t="n">
+      <c r="H6" s="63" t="n">
         <f aca="false">F6*G6</f>
         <v>48.895</v>
       </c>
-      <c r="I6" s="52" t="n">
+      <c r="I6" s="63" t="n">
         <f aca="false">G6/$B$3*1000</f>
         <v>0.57037037037037</v>
       </c>
-      <c r="J6" s="52" t="n">
+      <c r="J6" s="63" t="n">
         <f aca="false">F6*I6</f>
         <v>72.437037037037</v>
       </c>
-      <c r="K6" s="53" t="n">
+      <c r="K6" s="64" t="n">
         <v>7.7</v>
       </c>
-      <c r="L6" s="53" t="n">
+      <c r="L6" s="64" t="n">
         <f aca="false">F6*K6</f>
         <v>977.9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>156</v>
+        <v>131</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="62" t="n">
         <v>50</v>
       </c>
-      <c r="E7" s="51" t="n">
+      <c r="E7" s="62" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="51" t="n">
+      <c r="F7" s="62" t="n">
         <f aca="false">D7+E7</f>
         <v>51</v>
       </c>
-      <c r="G7" s="52" t="n">
+      <c r="G7" s="63" t="n">
         <v>0.527</v>
       </c>
-      <c r="H7" s="52" t="n">
+      <c r="H7" s="63" t="n">
         <f aca="false">F7*G7</f>
         <v>26.877</v>
       </c>
-      <c r="I7" s="52" t="n">
+      <c r="I7" s="63" t="n">
         <f aca="false">G7/$B$3*1000</f>
         <v>0.780740740740741</v>
       </c>
-      <c r="J7" s="52" t="n">
+      <c r="J7" s="63" t="n">
         <f aca="false">F7*I7</f>
         <v>39.8177777777778</v>
       </c>
-      <c r="K7" s="53" t="n">
+      <c r="K7" s="64" t="n">
         <v>10.53</v>
       </c>
-      <c r="L7" s="53" t="n">
+      <c r="L7" s="64" t="n">
         <f aca="false">F7*K7</f>
         <v>537.03</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>157</v>
+        <v>190</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>158</v>
+        <v>191</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="51" t="n">
+      <c r="D8" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="E8" s="51" t="n">
+      <c r="E8" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="51" t="n">
+      <c r="F8" s="62" t="n">
         <f aca="false">D8+E8</f>
         <v>20</v>
       </c>
-      <c r="G8" s="52" t="n">
+      <c r="G8" s="63" t="n">
         <v>0.675</v>
       </c>
-      <c r="H8" s="52" t="n">
+      <c r="H8" s="63" t="n">
         <f aca="false">F8*G8</f>
         <v>13.5</v>
       </c>
-      <c r="I8" s="52" t="n">
+      <c r="I8" s="63" t="n">
         <f aca="false">G8/$B$3*1000</f>
         <v>1</v>
       </c>
-      <c r="J8" s="52" t="n">
+      <c r="J8" s="63" t="n">
         <f aca="false">F8*I8</f>
         <v>20</v>
       </c>
-      <c r="K8" s="53" t="n">
+      <c r="K8" s="64" t="n">
         <v>13.5</v>
       </c>
-      <c r="L8" s="53" t="n">
+      <c r="L8" s="64" t="n">
         <f aca="false">F8*K8</f>
         <v>270</v>
       </c>
@@ -4081,24 +4849,24 @@
         <v>248</v>
       </c>
       <c r="G9" s="18"/>
-      <c r="H9" s="54" t="n">
+      <c r="H9" s="65" t="n">
         <f aca="false">SUM(H5:H8)</f>
         <v>106.822</v>
       </c>
       <c r="I9" s="18"/>
-      <c r="J9" s="54" t="n">
+      <c r="J9" s="65" t="n">
         <f aca="false">SUM(J5:J8)</f>
         <v>158.254814814815</v>
       </c>
       <c r="K9" s="18"/>
-      <c r="L9" s="55" t="n">
+      <c r="L9" s="66" t="n">
         <f aca="false">SUM(L5:L8)</f>
         <v>2135.93</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="B11" s="43"/>
       <c r="C11" s="43"/>
@@ -4114,7 +4882,7 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="45" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="B12" s="45"/>
       <c r="C12" s="45"/>
@@ -4130,7 +4898,7 @@
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="45" t="s">
-        <v>178</v>
+        <v>210</v>
       </c>
       <c r="B13" s="45"/>
       <c r="C13" s="45"/>
@@ -4146,7 +4914,7 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
-        <v>179</v>
+        <v>211</v>
       </c>
       <c r="B14" s="43"/>
       <c r="C14" s="43"/>
@@ -4177,7 +4945,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4193,338 +4961,338 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>212</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="56" t="s">
-        <v>181</v>
-      </c>
-      <c r="B3" s="56" t="s">
-        <v>182</v>
-      </c>
-      <c r="C3" s="56" t="s">
-        <v>183</v>
-      </c>
-      <c r="D3" s="56" t="s">
-        <v>184</v>
+      <c r="A3" s="67" t="s">
+        <v>213</v>
+      </c>
+      <c r="B3" s="67" t="s">
+        <v>214</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>215</v>
+      </c>
+      <c r="D3" s="67" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="57" t="n">
+      <c r="A4" s="68" t="n">
         <v>1</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="C4" s="58" t="s">
-        <v>186</v>
+        <v>217</v>
+      </c>
+      <c r="C4" s="69" t="s">
+        <v>218</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>187</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="57" t="n">
+      <c r="A5" s="68" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="59" t="s">
-        <v>188</v>
+      <c r="B5" s="70" t="s">
+        <v>220</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>189</v>
+        <v>221</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>190</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="57" t="n">
+      <c r="A6" s="68" t="n">
         <v>3</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>191</v>
+        <v>217</v>
+      </c>
+      <c r="C6" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>192</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="57" t="n">
+      <c r="A7" s="68" t="n">
         <v>4</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>193</v>
+        <v>217</v>
+      </c>
+      <c r="C7" s="69" t="s">
+        <v>225</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>194</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="57" t="n">
+      <c r="A8" s="68" t="n">
         <v>5</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="C8" s="58" t="s">
-        <v>195</v>
+        <v>217</v>
+      </c>
+      <c r="C8" s="69" t="s">
+        <v>227</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>196</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="57" t="n">
+      <c r="A9" s="68" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="60" t="s">
-        <v>197</v>
-      </c>
-      <c r="C9" s="58" t="s">
-        <v>198</v>
+      <c r="B9" s="71" t="s">
+        <v>229</v>
+      </c>
+      <c r="C9" s="69" t="s">
+        <v>230</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>199</v>
+        <v>231</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="57" t="n">
+      <c r="A10" s="68" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="60" t="s">
-        <v>197</v>
-      </c>
-      <c r="C10" s="58" t="s">
-        <v>200</v>
+      <c r="B10" s="71" t="s">
+        <v>229</v>
+      </c>
+      <c r="C10" s="69" t="s">
+        <v>232</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>201</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="57" t="n">
+      <c r="A11" s="68" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="60" t="s">
-        <v>197</v>
-      </c>
-      <c r="C11" s="58" t="s">
-        <v>202</v>
+      <c r="B11" s="71" t="s">
+        <v>229</v>
+      </c>
+      <c r="C11" s="69" t="s">
+        <v>234</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>203</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="57" t="n">
+      <c r="A12" s="68" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="60" t="s">
-        <v>197</v>
-      </c>
-      <c r="C12" s="58" t="s">
-        <v>204</v>
+      <c r="B12" s="71" t="s">
+        <v>229</v>
+      </c>
+      <c r="C12" s="69" t="s">
+        <v>236</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>205</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="57" t="n">
+      <c r="A13" s="68" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="59" t="s">
-        <v>188</v>
+      <c r="B13" s="70" t="s">
+        <v>220</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>206</v>
+        <v>238</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>207</v>
+        <v>239</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="57" t="n">
+      <c r="A14" s="68" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="59" t="s">
-        <v>188</v>
+      <c r="B14" s="70" t="s">
+        <v>220</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>208</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="78" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="57" t="n">
+      <c r="A15" s="68" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="59" t="s">
-        <v>188</v>
+      <c r="B15" s="70" t="s">
+        <v>220</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>209</v>
+        <v>241</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>210</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="57" t="n">
+      <c r="A16" s="68" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="59" t="s">
-        <v>188</v>
+      <c r="B16" s="70" t="s">
+        <v>220</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>211</v>
+        <v>243</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>212</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="57" t="n">
+      <c r="A17" s="68" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="59" t="s">
-        <v>213</v>
+      <c r="B17" s="70" t="s">
+        <v>245</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>214</v>
+        <v>246</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>215</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="57" t="n">
+      <c r="A18" s="68" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="59" t="s">
-        <v>213</v>
+      <c r="B18" s="70" t="s">
+        <v>245</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>216</v>
+        <v>248</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>217</v>
+        <v>249</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="57" t="n">
+      <c r="A19" s="68" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="59" t="s">
-        <v>213</v>
+      <c r="B19" s="70" t="s">
+        <v>245</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>218</v>
+        <v>250</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>219</v>
+        <v>251</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="57" t="n">
+      <c r="A20" s="68" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="59" t="s">
-        <v>213</v>
+      <c r="B20" s="70" t="s">
+        <v>245</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>220</v>
+        <v>252</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>221</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="61" t="s">
-        <v>222</v>
+      <c r="A22" s="72" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B23" s="63" t="s">
-        <v>224</v>
-      </c>
-      <c r="C23" s="63"/>
-      <c r="D23" s="63"/>
+      <c r="A23" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B23" s="74" t="s">
+        <v>256</v>
+      </c>
+      <c r="C23" s="74"/>
+      <c r="D23" s="74"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B24" s="63" t="s">
-        <v>225</v>
-      </c>
-      <c r="C24" s="63"/>
-      <c r="D24" s="63"/>
+      <c r="A24" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B24" s="74" t="s">
+        <v>257</v>
+      </c>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B25" s="63" t="s">
-        <v>226</v>
-      </c>
-      <c r="C25" s="63"/>
-      <c r="D25" s="63"/>
+      <c r="A25" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B25" s="74" t="s">
+        <v>258</v>
+      </c>
+      <c r="C25" s="74"/>
+      <c r="D25" s="74"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B26" s="63" t="s">
-        <v>227</v>
-      </c>
-      <c r="C26" s="63"/>
-      <c r="D26" s="63"/>
+      <c r="A26" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B26" s="74" t="s">
+        <v>259</v>
+      </c>
+      <c r="C26" s="74"/>
+      <c r="D26" s="74"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B27" s="63" t="s">
-        <v>228</v>
-      </c>
-      <c r="C27" s="63"/>
-      <c r="D27" s="63"/>
+      <c r="A27" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B27" s="74" t="s">
+        <v>260</v>
+      </c>
+      <c r="C27" s="74"/>
+      <c r="D27" s="74"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B28" s="63" t="s">
-        <v>229</v>
-      </c>
-      <c r="C28" s="63"/>
-      <c r="D28" s="63"/>
+      <c r="A28" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B28" s="74" t="s">
+        <v>261</v>
+      </c>
+      <c r="C28" s="74"/>
+      <c r="D28" s="74"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="62" t="s">
-        <v>223</v>
-      </c>
-      <c r="B29" s="63" t="s">
-        <v>230</v>
-      </c>
-      <c r="C29" s="63"/>
-      <c r="D29" s="63"/>
+      <c r="A29" s="73" t="s">
+        <v>255</v>
+      </c>
+      <c r="B29" s="74" t="s">
+        <v>262</v>
+      </c>
+      <c r="C29" s="74"/>
+      <c r="D29" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>